<commit_message>
PV2 discount rate rework, continued formula reformatting
</commit_message>
<xml_diff>
--- a/EconAutomation/src/supporting_docs/econ_wb_templates/WorkingCalc_Current.xlsx
+++ b/EconAutomation/src/supporting_docs/econ_wb_templates/WorkingCalc_Current.xlsx
@@ -12,7 +12,7 @@
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ACC5C77-3153-49AF-A98A-0B803BD0EF4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-75" windowWidth="29040" windowHeight="15720" tabRatio="808" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FDA883B1-89AA-41DF-A01F-246993B8D400}"/>
+    <workbookView xWindow="28680" yWindow="-75" windowWidth="29040" windowHeight="15720" xr2:uid="{FDA883B1-89AA-41DF-A01F-246993B8D400}"/>
   </bookViews>
   <sheets>
     <sheet name="REPORT_OUTPUTS" sheetId="30" r:id="rId1"/>
@@ -1463,10 +1463,10 @@
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
-    <numFmt numFmtId="167" formatCode="#0.0"/>
-    <numFmt numFmtId="168" formatCode="#0.000"/>
-    <numFmt numFmtId="169" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="#0.0"/>
+    <numFmt numFmtId="167" formatCode="#0.000"/>
+    <numFmt numFmtId="168" formatCode="0.000"/>
   </numFmts>
   <fonts count="21" x14ac:knownFonts="1">
     <font>
@@ -2221,7 +2221,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="135">
+  <cellXfs count="133">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2289,10 +2289,10 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="168" fontId="11" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -2323,13 +2323,13 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="167" fontId="13" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="168" fontId="13" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2400,7 +2400,7 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="19" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="19" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="19" fillId="0" borderId="23" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2444,8 +2444,40 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="2" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="3" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="19" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="29" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="29" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="11" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2467,6 +2499,9 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="13" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2494,45 +2529,6 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="2" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="3" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="3" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="166" fontId="19" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="29" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="18" fillId="18" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="29" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="3" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -2541,6 +2537,76 @@
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="116">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -2653,76 +2719,6 @@
         <family val="1"/>
         <scheme val="none"/>
       </font>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
@@ -5624,11 +5620,11 @@
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{32BFE16E-A259-4C63-8DCF-00C9A6EFA78D}" name="Table15" displayName="Table15" ref="F1:G32" totalsRowShown="0" headerRowDxfId="3" dataDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{32BFE16E-A259-4C63-8DCF-00C9A6EFA78D}" name="Table15" displayName="Table15" ref="F1:G32" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="F1:G32" xr:uid="{32BFE16E-A259-4C63-8DCF-00C9A6EFA78D}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{099144D5-37E0-4580-8BDC-BF9DA5901655}" name="PASTED YEAR" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{DEBA212E-45CC-4A41-A95A-1A261BC6D9AB}" name="PASTED DISCOUNT RATES" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{099144D5-37E0-4580-8BDC-BF9DA5901655}" name="PASTED YEAR" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{DEBA212E-45CC-4A41-A95A-1A261BC6D9AB}" name="PASTED DISCOUNT RATES" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6108,24 +6104,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="99" t="s">
+      <c r="A1" s="115" t="s">
         <v>304</v>
       </c>
-      <c r="B1" s="100"/>
-      <c r="C1" s="100"/>
-      <c r="D1" s="101"/>
+      <c r="B1" s="116"/>
+      <c r="C1" s="116"/>
+      <c r="D1" s="117"/>
       <c r="E1" s="56"/>
-      <c r="F1" s="102" t="str" cm="1">
+      <c r="F1" s="118" t="str" cm="1">
         <f t="array" aca="1" ref="F1" ca="1">_xlfn.TEXTAFTER(_xlfn.TEXTBEFORE(CELL("filename",A1),"]"),"[") &amp; " TABLES"</f>
         <v>WorkingCalc_Current.xlsx TABLES</v>
       </c>
-      <c r="G1" s="103"/>
+      <c r="G1" s="119"/>
       <c r="H1" s="56"/>
-      <c r="I1" s="104" t="str" cm="1">
+      <c r="I1" s="120" t="str" cm="1">
         <f t="array" aca="1" ref="I1" ca="1">_xlfn.TEXTAFTER(_xlfn.TEXTBEFORE(CELL("filename",D1),"]"),"[") &amp; " CHARTS"</f>
         <v>WorkingCalc_Current.xlsx CHARTS</v>
       </c>
-      <c r="J1" s="105"/>
+      <c r="J1" s="121"/>
     </row>
     <row r="2" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="57" t="s">
@@ -6238,7 +6234,7 @@
       <c r="J6" s="76"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="130" t="s">
+      <c r="A7" s="110" t="s">
         <v>323</v>
       </c>
       <c r="B7" s="72" t="s">
@@ -6257,7 +6253,7 @@
       <c r="J7" s="80"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="126" t="s">
+      <c r="A8" s="106" t="s">
         <v>325</v>
       </c>
       <c r="B8" s="72" t="s">
@@ -6276,7 +6272,7 @@
       <c r="J8" s="76"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="130" t="s">
+      <c r="A9" s="110" t="s">
         <v>326</v>
       </c>
       <c r="B9" s="72" t="s">
@@ -6285,7 +6281,7 @@
       <c r="C9" s="72" t="s">
         <v>415</v>
       </c>
-      <c r="D9" s="123" cm="1">
+      <c r="D9" s="103" cm="1">
         <f t="array" aca="1" ref="D9" ca="1">IF(OR(IF(OR(A9="", B9="", C9=""), "", INDIRECT("'" &amp; B9 &amp; "'!" &amp; C9))=0, IF(OR(A9="", B9="", C9=""), "", INDIRECT("'" &amp; B9 &amp; "'!" &amp; C9))=""),"",INDIRECT("'" &amp; B9 &amp; "'!" &amp; C9))</f>
         <v>2.0736944174645666E-2</v>
       </c>
@@ -6295,16 +6291,16 @@
       <c r="J9" s="80"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="127" t="s">
+      <c r="A10" s="107" t="s">
         <v>327</v>
       </c>
-      <c r="B10" s="124" t="s">
+      <c r="B10" s="104" t="s">
         <v>324</v>
       </c>
-      <c r="C10" s="125" t="s">
+      <c r="C10" s="105" t="s">
         <v>416</v>
       </c>
-      <c r="D10" s="123" t="str" cm="1">
+      <c r="D10" s="103" t="str" cm="1">
         <f t="array" aca="1" ref="D10" ca="1">IF(OR(IF(OR(A10="", B10="", C10=""), "", INDIRECT("'" &amp; B10 &amp; "'!" &amp; C10))=0, IF(OR(A10="", B10="", C10=""), "", INDIRECT("'" &amp; B10 &amp; "'!" &amp; C10))=""),"",INDIRECT("'" &amp; B10 &amp; "'!" &amp; C10))</f>
         <v/>
       </c>
@@ -6314,16 +6310,16 @@
       <c r="J10" s="76"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="131" t="s">
+      <c r="A11" s="111" t="s">
         <v>328</v>
       </c>
-      <c r="B11" s="124" t="s">
+      <c r="B11" s="104" t="s">
         <v>324</v>
       </c>
-      <c r="C11" s="125" t="s">
+      <c r="C11" s="105" t="s">
         <v>417</v>
       </c>
-      <c r="D11" s="123" cm="1">
+      <c r="D11" s="103" cm="1">
         <f t="array" aca="1" ref="D11" ca="1">IF(OR(IF(OR(A11="", B11="", C11=""), "", INDIRECT("'" &amp; B11 &amp; "'!" &amp; C11))=0, IF(OR(A11="", B11="", C11=""), "", INDIRECT("'" &amp; B11 &amp; "'!" &amp; C11))=""),"",INDIRECT("'" &amp; B11 &amp; "'!" &amp; C11))</f>
         <v>3.5117348400309334E-2</v>
       </c>
@@ -6333,16 +6329,16 @@
       <c r="J11" s="80"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="127" t="s">
+      <c r="A12" s="107" t="s">
         <v>329</v>
       </c>
-      <c r="B12" s="124" t="s">
+      <c r="B12" s="104" t="s">
         <v>324</v>
       </c>
-      <c r="C12" s="125" t="s">
+      <c r="C12" s="105" t="s">
         <v>418</v>
       </c>
-      <c r="D12" s="123" t="str" cm="1">
+      <c r="D12" s="103" t="str" cm="1">
         <f t="array" aca="1" ref="D12" ca="1">IF(OR(IF(OR(A12="", B12="", C12=""), "", INDIRECT("'" &amp; B12 &amp; "'!" &amp; C12))=0, IF(OR(A12="", B12="", C12=""), "", INDIRECT("'" &amp; B12 &amp; "'!" &amp; C12))=""),"",INDIRECT("'" &amp; B12 &amp; "'!" &amp; C12))</f>
         <v/>
       </c>
@@ -6352,16 +6348,16 @@
       <c r="J12" s="76"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="131" t="s">
+      <c r="A13" s="111" t="s">
         <v>330</v>
       </c>
-      <c r="B13" s="124" t="s">
+      <c r="B13" s="104" t="s">
         <v>324</v>
       </c>
-      <c r="C13" s="125" t="s">
+      <c r="C13" s="105" t="s">
         <v>419</v>
       </c>
-      <c r="D13" s="123" cm="1">
+      <c r="D13" s="103" cm="1">
         <f t="array" aca="1" ref="D13" ca="1">IF(OR(IF(OR(A13="", B13="", C13=""), "", INDIRECT("'" &amp; B13 &amp; "'!" &amp; C13))=0, IF(OR(A13="", B13="", C13=""), "", INDIRECT("'" &amp; B13 &amp; "'!" &amp; C13))=""),"",INDIRECT("'" &amp; B13 &amp; "'!" &amp; C13))</f>
         <v>2.9548225004298212E-2</v>
       </c>
@@ -6371,16 +6367,16 @@
       <c r="J13" s="80"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="128" t="s">
+      <c r="A14" s="108" t="s">
         <v>331</v>
       </c>
-      <c r="B14" s="124" t="s">
+      <c r="B14" s="104" t="s">
         <v>324</v>
       </c>
-      <c r="C14" s="125" t="s">
+      <c r="C14" s="105" t="s">
         <v>420</v>
       </c>
-      <c r="D14" s="123" t="str" cm="1">
+      <c r="D14" s="103" t="str" cm="1">
         <f t="array" aca="1" ref="D14" ca="1">IF(OR(IF(OR(A14="", B14="", C14=""), "", INDIRECT("'" &amp; B14 &amp; "'!" &amp; C14))=0, IF(OR(A14="", B14="", C14=""), "", INDIRECT("'" &amp; B14 &amp; "'!" &amp; C14))=""),"",INDIRECT("'" &amp; B14 &amp; "'!" &amp; C14))</f>
         <v/>
       </c>
@@ -6390,16 +6386,16 @@
       <c r="J14" s="76"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="131" t="s">
+      <c r="A15" s="111" t="s">
         <v>332</v>
       </c>
-      <c r="B15" s="124" t="s">
+      <c r="B15" s="104" t="s">
         <v>324</v>
       </c>
-      <c r="C15" s="125" t="s">
+      <c r="C15" s="105" t="s">
         <v>421</v>
       </c>
-      <c r="D15" s="123" cm="1">
+      <c r="D15" s="103" cm="1">
         <f t="array" aca="1" ref="D15" ca="1">IF(OR(IF(OR(A15="", B15="", C15=""), "", INDIRECT("'" &amp; B15 &amp; "'!" &amp; C15))=0, IF(OR(A15="", B15="", C15=""), "", INDIRECT("'" &amp; B15 &amp; "'!" &amp; C15))=""),"",INDIRECT("'" &amp; B15 &amp; "'!" &amp; C15))</f>
         <v>6.3201478284775625E-3</v>
       </c>
@@ -6409,16 +6405,16 @@
       <c r="J15" s="80"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="128" t="s">
+      <c r="A16" s="108" t="s">
         <v>333</v>
       </c>
-      <c r="B16" s="124" t="s">
+      <c r="B16" s="104" t="s">
         <v>324</v>
       </c>
-      <c r="C16" s="125" t="s">
+      <c r="C16" s="105" t="s">
         <v>422</v>
       </c>
-      <c r="D16" s="123" t="str" cm="1">
+      <c r="D16" s="103" t="str" cm="1">
         <f t="array" aca="1" ref="D16" ca="1">IF(OR(IF(OR(A16="", B16="", C16=""), "", INDIRECT("'" &amp; B16 &amp; "'!" &amp; C16))=0, IF(OR(A16="", B16="", C16=""), "", INDIRECT("'" &amp; B16 &amp; "'!" &amp; C16))=""),"",INDIRECT("'" &amp; B16 &amp; "'!" &amp; C16))</f>
         <v/>
       </c>
@@ -6428,16 +6424,16 @@
       <c r="J16" s="76"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" s="131" t="s">
+      <c r="A17" s="111" t="s">
         <v>334</v>
       </c>
-      <c r="B17" s="124" t="s">
+      <c r="B17" s="104" t="s">
         <v>324</v>
       </c>
-      <c r="C17" s="125" t="s">
+      <c r="C17" s="105" t="s">
         <v>423</v>
       </c>
-      <c r="D17" s="123" cm="1">
+      <c r="D17" s="103" cm="1">
         <f t="array" aca="1" ref="D17" ca="1">IF(OR(IF(OR(A17="", B17="", C17=""), "", INDIRECT("'" &amp; B17 &amp; "'!" &amp; C17))=0, IF(OR(A17="", B17="", C17=""), "", INDIRECT("'" &amp; B17 &amp; "'!" &amp; C17))=""),"",INDIRECT("'" &amp; B17 &amp; "'!" &amp; C17))</f>
         <v>2.5219757035239265E-2</v>
       </c>
@@ -6447,16 +6443,16 @@
       <c r="J17" s="80"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="128" t="s">
+      <c r="A18" s="108" t="s">
         <v>335</v>
       </c>
-      <c r="B18" s="124" t="s">
+      <c r="B18" s="104" t="s">
         <v>324</v>
       </c>
-      <c r="C18" s="125" t="s">
+      <c r="C18" s="105" t="s">
         <v>424</v>
       </c>
-      <c r="D18" s="123" t="str" cm="1">
+      <c r="D18" s="103" t="str" cm="1">
         <f t="array" aca="1" ref="D18" ca="1">IF(OR(IF(OR(A18="", B18="", C18=""), "", INDIRECT("'" &amp; B18 &amp; "'!" &amp; C18))=0, IF(OR(A18="", B18="", C18=""), "", INDIRECT("'" &amp; B18 &amp; "'!" &amp; C18))=""),"",INDIRECT("'" &amp; B18 &amp; "'!" &amp; C18))</f>
         <v/>
       </c>
@@ -6466,16 +6462,16 @@
       <c r="J18" s="76"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="131" t="s">
+      <c r="A19" s="111" t="s">
         <v>336</v>
       </c>
-      <c r="B19" s="124" t="s">
+      <c r="B19" s="104" t="s">
         <v>324</v>
       </c>
-      <c r="C19" s="125" t="s">
+      <c r="C19" s="105" t="s">
         <v>425</v>
       </c>
-      <c r="D19" s="123" cm="1">
+      <c r="D19" s="103" cm="1">
         <f t="array" aca="1" ref="D19" ca="1">IF(OR(IF(OR(A19="", B19="", C19=""), "", INDIRECT("'" &amp; B19 &amp; "'!" &amp; C19))=0, IF(OR(A19="", B19="", C19=""), "", INDIRECT("'" &amp; B19 &amp; "'!" &amp; C19))=""),"",INDIRECT("'" &amp; B19 &amp; "'!" &amp; C19))</f>
         <v>5.2913605158896315E-2</v>
       </c>
@@ -6485,16 +6481,16 @@
       <c r="J19" s="80"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" s="128" t="s">
+      <c r="A20" s="108" t="s">
         <v>337</v>
       </c>
-      <c r="B20" s="124" t="s">
+      <c r="B20" s="104" t="s">
         <v>324</v>
       </c>
-      <c r="C20" s="125" t="s">
+      <c r="C20" s="105" t="s">
         <v>426</v>
       </c>
-      <c r="D20" s="123" t="str" cm="1">
+      <c r="D20" s="103" t="str" cm="1">
         <f t="array" aca="1" ref="D20" ca="1">IF(OR(IF(OR(A20="", B20="", C20=""), "", INDIRECT("'" &amp; B20 &amp; "'!" &amp; C20))=0, IF(OR(A20="", B20="", C20=""), "", INDIRECT("'" &amp; B20 &amp; "'!" &amp; C20))=""),"",INDIRECT("'" &amp; B20 &amp; "'!" &amp; C20))</f>
         <v/>
       </c>
@@ -6504,16 +6500,16 @@
       <c r="J20" s="76"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A21" s="131" t="s">
+      <c r="A21" s="111" t="s">
         <v>338</v>
       </c>
-      <c r="B21" s="124" t="s">
+      <c r="B21" s="104" t="s">
         <v>324</v>
       </c>
-      <c r="C21" s="125" t="s">
+      <c r="C21" s="105" t="s">
         <v>427</v>
       </c>
-      <c r="D21" s="123" cm="1">
+      <c r="D21" s="103" cm="1">
         <f t="array" aca="1" ref="D21" ca="1">IF(OR(IF(OR(A21="", B21="", C21=""), "", INDIRECT("'" &amp; B21 &amp; "'!" &amp; C21))=0, IF(OR(A21="", B21="", C21=""), "", INDIRECT("'" &amp; B21 &amp; "'!" &amp; C21))=""),"",INDIRECT("'" &amp; B21 &amp; "'!" &amp; C21))</f>
         <v>5.2018836646548605E-2</v>
       </c>
@@ -6523,16 +6519,16 @@
       <c r="J21" s="80"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" s="128" t="s">
+      <c r="A22" s="108" t="s">
         <v>339</v>
       </c>
-      <c r="B22" s="124" t="s">
+      <c r="B22" s="104" t="s">
         <v>324</v>
       </c>
-      <c r="C22" s="125" t="s">
+      <c r="C22" s="105" t="s">
         <v>428</v>
       </c>
-      <c r="D22" s="123" t="str" cm="1">
+      <c r="D22" s="103" t="str" cm="1">
         <f t="array" aca="1" ref="D22" ca="1">IF(OR(IF(OR(A22="", B22="", C22=""), "", INDIRECT("'" &amp; B22 &amp; "'!" &amp; C22))=0, IF(OR(A22="", B22="", C22=""), "", INDIRECT("'" &amp; B22 &amp; "'!" &amp; C22))=""),"",INDIRECT("'" &amp; B22 &amp; "'!" &amp; C22))</f>
         <v/>
       </c>
@@ -6542,16 +6538,16 @@
       <c r="J22" s="76"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" s="131" t="s">
+      <c r="A23" s="111" t="s">
         <v>340</v>
       </c>
-      <c r="B23" s="124" t="s">
+      <c r="B23" s="104" t="s">
         <v>324</v>
       </c>
-      <c r="C23" s="125" t="s">
+      <c r="C23" s="105" t="s">
         <v>429</v>
       </c>
-      <c r="D23" s="123" cm="1">
+      <c r="D23" s="103" cm="1">
         <f t="array" aca="1" ref="D23" ca="1">IF(OR(IF(OR(A23="", B23="", C23=""), "", INDIRECT("'" &amp; B23 &amp; "'!" &amp; C23))=0, IF(OR(A23="", B23="", C23=""), "", INDIRECT("'" &amp; B23 &amp; "'!" &amp; C23))=""),"",INDIRECT("'" &amp; B23 &amp; "'!" &amp; C23))</f>
         <v>5.2900906226266198E-2</v>
       </c>
@@ -6561,7 +6557,7 @@
       <c r="J23" s="80"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" s="129" t="s">
+      <c r="A24" s="109" t="s">
         <v>341</v>
       </c>
       <c r="B24" s="65" t="s">
@@ -6580,7 +6576,7 @@
       <c r="J24" s="76"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A25" s="130" t="s">
+      <c r="A25" s="110" t="s">
         <v>342</v>
       </c>
       <c r="B25" s="72" t="s">
@@ -6599,7 +6595,7 @@
       <c r="J25" s="80"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A26" s="126" t="s">
+      <c r="A26" s="106" t="s">
         <v>343</v>
       </c>
       <c r="B26" s="72" t="s">
@@ -7763,22 +7759,22 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:G2 A6:G114">
-    <cfRule type="expression" dxfId="13" priority="1">
+    <cfRule type="expression" dxfId="9" priority="1">
       <formula>OR($C2=0, $A2="Header")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:G6">
-    <cfRule type="expression" dxfId="12" priority="2">
+    <cfRule type="expression" dxfId="8" priority="2">
       <formula>$A2=Header</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:XFD32">
-    <cfRule type="expression" dxfId="11" priority="18">
+    <cfRule type="expression" dxfId="7" priority="18">
       <formula>#REF!=Header</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H33:XFD33">
-    <cfRule type="expression" dxfId="10" priority="17">
+    <cfRule type="expression" dxfId="6" priority="17">
       <formula>$A6=Header</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10127,26 +10123,26 @@
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="I1:L1 B1:G6 E8:G25 D8:D26">
-    <cfRule type="expression" dxfId="9" priority="5">
+    <cfRule type="expression" dxfId="5" priority="5">
       <formula>$C1=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="6">
+    <cfRule type="expression" dxfId="4" priority="6">
       <formula>$C1=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:L18">
-    <cfRule type="expression" dxfId="7" priority="11">
+    <cfRule type="expression" dxfId="3" priority="11">
       <formula>#REF!=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="12">
+    <cfRule type="expression" dxfId="2" priority="12">
       <formula>#REF!=1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I19:L19">
-    <cfRule type="expression" dxfId="5" priority="9">
+    <cfRule type="expression" dxfId="1" priority="9">
       <formula>$C6=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="10">
+    <cfRule type="expression" dxfId="0" priority="10">
       <formula>$C6=1</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12276,10 +12272,10 @@
       <c r="C1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="122" t="s">
+      <c r="F1" s="102" t="s">
         <v>411</v>
       </c>
-      <c r="G1" s="122" t="s">
+      <c r="G1" s="102" t="s">
         <v>412</v>
       </c>
     </row>
@@ -12293,8 +12289,8 @@
       <c r="C2" s="40" t="s">
         <v>266</v>
       </c>
-      <c r="F2" s="132"/>
-      <c r="G2" s="132"/>
+      <c r="F2" s="112"/>
+      <c r="G2" s="112"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -12306,8 +12302,8 @@
       <c r="C3" s="40" t="s">
         <v>267</v>
       </c>
-      <c r="F3" s="133"/>
-      <c r="G3" s="132"/>
+      <c r="F3" s="113"/>
+      <c r="G3" s="112"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -12319,8 +12315,8 @@
       <c r="C4" s="40" t="s">
         <v>268</v>
       </c>
-      <c r="F4" s="133"/>
-      <c r="G4" s="132"/>
+      <c r="F4" s="113"/>
+      <c r="G4" s="112"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
@@ -12332,8 +12328,8 @@
       <c r="C5" s="40" t="s">
         <v>269</v>
       </c>
-      <c r="F5" s="133"/>
-      <c r="G5" s="132"/>
+      <c r="F5" s="113"/>
+      <c r="G5" s="112"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
@@ -12345,8 +12341,8 @@
       <c r="C6" s="40" t="s">
         <v>270</v>
       </c>
-      <c r="F6" s="133"/>
-      <c r="G6" s="132"/>
+      <c r="F6" s="113"/>
+      <c r="G6" s="112"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
@@ -12358,8 +12354,8 @@
       <c r="C7" s="40" t="s">
         <v>271</v>
       </c>
-      <c r="F7" s="133"/>
-      <c r="G7" s="132"/>
+      <c r="F7" s="113"/>
+      <c r="G7" s="112"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
@@ -12371,8 +12367,8 @@
       <c r="C8" s="40" t="s">
         <v>272</v>
       </c>
-      <c r="F8" s="133"/>
-      <c r="G8" s="132"/>
+      <c r="F8" s="113"/>
+      <c r="G8" s="112"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
@@ -12384,8 +12380,8 @@
       <c r="C9" s="40" t="s">
         <v>273</v>
       </c>
-      <c r="F9" s="133"/>
-      <c r="G9" s="132"/>
+      <c r="F9" s="113"/>
+      <c r="G9" s="112"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
@@ -12397,8 +12393,8 @@
       <c r="C10" s="40" t="s">
         <v>274</v>
       </c>
-      <c r="F10" s="133"/>
-      <c r="G10" s="132"/>
+      <c r="F10" s="113"/>
+      <c r="G10" s="112"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
@@ -12410,8 +12406,8 @@
       <c r="C11" s="40" t="s">
         <v>275</v>
       </c>
-      <c r="F11" s="133"/>
-      <c r="G11" s="132"/>
+      <c r="F11" s="113"/>
+      <c r="G11" s="112"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
@@ -12423,8 +12419,8 @@
       <c r="C12" s="40" t="s">
         <v>276</v>
       </c>
-      <c r="F12" s="133"/>
-      <c r="G12" s="132"/>
+      <c r="F12" s="113"/>
+      <c r="G12" s="112"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
@@ -12436,8 +12432,8 @@
       <c r="C13" s="40" t="s">
         <v>277</v>
       </c>
-      <c r="F13" s="133"/>
-      <c r="G13" s="132"/>
+      <c r="F13" s="113"/>
+      <c r="G13" s="112"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
@@ -12449,8 +12445,8 @@
       <c r="C14" s="40" t="s">
         <v>278</v>
       </c>
-      <c r="F14" s="133"/>
-      <c r="G14" s="132"/>
+      <c r="F14" s="113"/>
+      <c r="G14" s="112"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
@@ -12462,8 +12458,8 @@
       <c r="C15" s="40" t="s">
         <v>279</v>
       </c>
-      <c r="F15" s="133"/>
-      <c r="G15" s="132"/>
+      <c r="F15" s="113"/>
+      <c r="G15" s="112"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
@@ -12475,8 +12471,8 @@
       <c r="C16" s="40" t="s">
         <v>280</v>
       </c>
-      <c r="F16" s="133"/>
-      <c r="G16" s="132"/>
+      <c r="F16" s="113"/>
+      <c r="G16" s="112"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
@@ -12488,8 +12484,8 @@
       <c r="C17" s="40" t="s">
         <v>281</v>
       </c>
-      <c r="F17" s="133"/>
-      <c r="G17" s="132"/>
+      <c r="F17" s="113"/>
+      <c r="G17" s="112"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
@@ -12501,8 +12497,8 @@
       <c r="C18" s="40" t="s">
         <v>282</v>
       </c>
-      <c r="F18" s="133"/>
-      <c r="G18" s="132"/>
+      <c r="F18" s="113"/>
+      <c r="G18" s="112"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
@@ -12514,8 +12510,8 @@
       <c r="C19" s="40" t="s">
         <v>283</v>
       </c>
-      <c r="F19" s="133"/>
-      <c r="G19" s="132"/>
+      <c r="F19" s="113"/>
+      <c r="G19" s="112"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
@@ -12527,8 +12523,8 @@
       <c r="C20" s="40" t="s">
         <v>284</v>
       </c>
-      <c r="F20" s="133"/>
-      <c r="G20" s="132"/>
+      <c r="F20" s="113"/>
+      <c r="G20" s="112"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
@@ -12540,8 +12536,8 @@
       <c r="C21" s="40" t="s">
         <v>285</v>
       </c>
-      <c r="F21" s="133"/>
-      <c r="G21" s="132"/>
+      <c r="F21" s="113"/>
+      <c r="G21" s="112"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
@@ -12553,8 +12549,8 @@
       <c r="C22" s="40" t="s">
         <v>286</v>
       </c>
-      <c r="F22" s="133"/>
-      <c r="G22" s="132"/>
+      <c r="F22" s="113"/>
+      <c r="G22" s="112"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
@@ -12566,8 +12562,8 @@
       <c r="C23" s="40" t="s">
         <v>287</v>
       </c>
-      <c r="F23" s="133"/>
-      <c r="G23" s="132"/>
+      <c r="F23" s="113"/>
+      <c r="G23" s="112"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
@@ -12579,8 +12575,8 @@
       <c r="C24" s="40" t="s">
         <v>288</v>
       </c>
-      <c r="F24" s="133"/>
-      <c r="G24" s="132"/>
+      <c r="F24" s="113"/>
+      <c r="G24" s="112"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
@@ -12592,8 +12588,8 @@
       <c r="C25" s="40" t="s">
         <v>289</v>
       </c>
-      <c r="F25" s="133"/>
-      <c r="G25" s="132"/>
+      <c r="F25" s="113"/>
+      <c r="G25" s="112"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
@@ -12605,8 +12601,8 @@
       <c r="C26" s="40" t="s">
         <v>290</v>
       </c>
-      <c r="F26" s="133"/>
-      <c r="G26" s="132"/>
+      <c r="F26" s="113"/>
+      <c r="G26" s="112"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
@@ -12618,8 +12614,8 @@
       <c r="C27" s="40" t="s">
         <v>291</v>
       </c>
-      <c r="F27" s="133"/>
-      <c r="G27" s="132"/>
+      <c r="F27" s="113"/>
+      <c r="G27" s="112"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
@@ -12631,8 +12627,8 @@
       <c r="C28" s="40" t="s">
         <v>292</v>
       </c>
-      <c r="F28" s="133"/>
-      <c r="G28" s="132"/>
+      <c r="F28" s="113"/>
+      <c r="G28" s="112"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
@@ -12644,8 +12640,8 @@
       <c r="C29" s="40" t="s">
         <v>293</v>
       </c>
-      <c r="F29" s="133"/>
-      <c r="G29" s="132"/>
+      <c r="F29" s="113"/>
+      <c r="G29" s="112"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
@@ -12657,8 +12653,8 @@
       <c r="C30" s="40" t="s">
         <v>294</v>
       </c>
-      <c r="F30" s="133"/>
-      <c r="G30" s="132"/>
+      <c r="F30" s="113"/>
+      <c r="G30" s="112"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
@@ -12670,12 +12666,12 @@
       <c r="C31" s="40" t="s">
         <v>295</v>
       </c>
-      <c r="F31" s="133"/>
-      <c r="G31" s="132"/>
+      <c r="F31" s="113"/>
+      <c r="G31" s="112"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="F32" s="133"/>
-      <c r="G32" s="134"/>
+      <c r="F32" s="113"/>
+      <c r="G32" s="114"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -15368,10 +15364,10 @@
       </c>
     </row>
     <row r="91" spans="10:11" x14ac:dyDescent="0.25">
-      <c r="J91" s="98" t="s">
+      <c r="J91" s="122" t="s">
         <v>31</v>
       </c>
-      <c r="K91" s="98"/>
+      <c r="K91" s="122"/>
     </row>
     <row r="92" spans="10:11" ht="49.5" x14ac:dyDescent="0.25">
       <c r="J92" s="10" t="s">
@@ -17070,14 +17066,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:160" x14ac:dyDescent="0.25">
-      <c r="B1" s="108" t="s">
+      <c r="B1" s="125" t="s">
         <v>223</v>
       </c>
-      <c r="C1" s="107"/>
-      <c r="D1" s="107"/>
-      <c r="E1" s="107"/>
-      <c r="F1" s="107"/>
-      <c r="G1" s="107"/>
+      <c r="C1" s="124"/>
+      <c r="D1" s="124"/>
+      <c r="E1" s="124"/>
+      <c r="F1" s="124"/>
+      <c r="G1" s="124"/>
       <c r="H1" s="49"/>
       <c r="I1" s="49"/>
       <c r="J1" s="49"/>
@@ -17087,14 +17083,14 @@
       <c r="N1" s="49"/>
       <c r="O1" s="49"/>
       <c r="P1" s="49"/>
-      <c r="R1" s="111" t="s">
+      <c r="R1" s="128" t="s">
         <v>223</v>
       </c>
-      <c r="S1" s="112"/>
-      <c r="T1" s="112"/>
-      <c r="U1" s="112"/>
-      <c r="V1" s="112"/>
-      <c r="W1" s="112"/>
+      <c r="S1" s="129"/>
+      <c r="T1" s="129"/>
+      <c r="U1" s="129"/>
+      <c r="V1" s="129"/>
+      <c r="W1" s="129"/>
       <c r="X1" s="34"/>
       <c r="Y1" s="34"/>
       <c r="Z1" s="34"/>
@@ -17104,14 +17100,14 @@
       <c r="AD1" s="34"/>
       <c r="AE1" s="34"/>
       <c r="AF1" s="34"/>
-      <c r="AH1" s="108" t="s">
+      <c r="AH1" s="125" t="s">
         <v>223</v>
       </c>
-      <c r="AI1" s="107"/>
-      <c r="AJ1" s="107"/>
-      <c r="AK1" s="107"/>
-      <c r="AL1" s="107"/>
-      <c r="AM1" s="107"/>
+      <c r="AI1" s="124"/>
+      <c r="AJ1" s="124"/>
+      <c r="AK1" s="124"/>
+      <c r="AL1" s="124"/>
+      <c r="AM1" s="124"/>
       <c r="AN1" s="49"/>
       <c r="AO1" s="49"/>
       <c r="AP1" s="49"/>
@@ -17121,14 +17117,14 @@
       <c r="AT1" s="49"/>
       <c r="AU1" s="49"/>
       <c r="AV1" s="49"/>
-      <c r="AX1" s="108" t="s">
+      <c r="AX1" s="125" t="s">
         <v>223</v>
       </c>
-      <c r="AY1" s="107"/>
-      <c r="AZ1" s="107"/>
-      <c r="BA1" s="107"/>
-      <c r="BB1" s="107"/>
-      <c r="BC1" s="107"/>
+      <c r="AY1" s="124"/>
+      <c r="AZ1" s="124"/>
+      <c r="BA1" s="124"/>
+      <c r="BB1" s="124"/>
+      <c r="BC1" s="124"/>
       <c r="BD1" s="49"/>
       <c r="BE1" s="49"/>
       <c r="BF1" s="49"/>
@@ -17138,14 +17134,14 @@
       <c r="BJ1" s="49"/>
       <c r="BK1" s="49"/>
       <c r="BL1" s="49"/>
-      <c r="BN1" s="108" t="s">
+      <c r="BN1" s="125" t="s">
         <v>223</v>
       </c>
-      <c r="BO1" s="107"/>
-      <c r="BP1" s="107"/>
-      <c r="BQ1" s="107"/>
-      <c r="BR1" s="107"/>
-      <c r="BS1" s="107"/>
+      <c r="BO1" s="124"/>
+      <c r="BP1" s="124"/>
+      <c r="BQ1" s="124"/>
+      <c r="BR1" s="124"/>
+      <c r="BS1" s="124"/>
       <c r="BT1" s="49"/>
       <c r="BU1" s="49"/>
       <c r="BV1" s="49"/>
@@ -17156,14 +17152,14 @@
       <c r="CA1" s="49"/>
       <c r="CB1" s="49"/>
       <c r="CC1" s="34"/>
-      <c r="CD1" s="108" t="s">
+      <c r="CD1" s="125" t="s">
         <v>223</v>
       </c>
-      <c r="CE1" s="107"/>
-      <c r="CF1" s="107"/>
-      <c r="CG1" s="107"/>
-      <c r="CH1" s="107"/>
-      <c r="CI1" s="107"/>
+      <c r="CE1" s="124"/>
+      <c r="CF1" s="124"/>
+      <c r="CG1" s="124"/>
+      <c r="CH1" s="124"/>
+      <c r="CI1" s="124"/>
       <c r="CJ1" s="49"/>
       <c r="CK1" s="49"/>
       <c r="CL1" s="49"/>
@@ -17173,14 +17169,14 @@
       <c r="CP1" s="49"/>
       <c r="CQ1" s="49"/>
       <c r="CR1" s="49"/>
-      <c r="CT1" s="108" t="s">
+      <c r="CT1" s="125" t="s">
         <v>223</v>
       </c>
-      <c r="CU1" s="107"/>
-      <c r="CV1" s="107"/>
-      <c r="CW1" s="107"/>
-      <c r="CX1" s="107"/>
-      <c r="CY1" s="107"/>
+      <c r="CU1" s="124"/>
+      <c r="CV1" s="124"/>
+      <c r="CW1" s="124"/>
+      <c r="CX1" s="124"/>
+      <c r="CY1" s="124"/>
       <c r="CZ1" s="49"/>
       <c r="DA1" s="49"/>
       <c r="DB1" s="49"/>
@@ -17190,14 +17186,14 @@
       <c r="DF1" s="49"/>
       <c r="DG1" s="49"/>
       <c r="DH1" s="49"/>
-      <c r="DJ1" s="108" t="s">
+      <c r="DJ1" s="125" t="s">
         <v>223</v>
       </c>
-      <c r="DK1" s="107"/>
-      <c r="DL1" s="107"/>
-      <c r="DM1" s="107"/>
-      <c r="DN1" s="107"/>
-      <c r="DO1" s="107"/>
+      <c r="DK1" s="124"/>
+      <c r="DL1" s="124"/>
+      <c r="DM1" s="124"/>
+      <c r="DN1" s="124"/>
+      <c r="DO1" s="124"/>
       <c r="DP1" s="49"/>
       <c r="DQ1" s="49"/>
       <c r="DR1" s="49"/>
@@ -17207,14 +17203,14 @@
       <c r="DV1" s="49"/>
       <c r="DW1" s="49"/>
       <c r="DX1" s="49"/>
-      <c r="DZ1" s="108" t="s">
+      <c r="DZ1" s="125" t="s">
         <v>223</v>
       </c>
-      <c r="EA1" s="107"/>
-      <c r="EB1" s="107"/>
-      <c r="EC1" s="107"/>
-      <c r="ED1" s="107"/>
-      <c r="EE1" s="107"/>
+      <c r="EA1" s="124"/>
+      <c r="EB1" s="124"/>
+      <c r="EC1" s="124"/>
+      <c r="ED1" s="124"/>
+      <c r="EE1" s="124"/>
       <c r="EF1" s="49"/>
       <c r="EG1" s="49"/>
       <c r="EH1" s="49"/>
@@ -17224,14 +17220,14 @@
       <c r="EL1" s="49"/>
       <c r="EM1" s="49"/>
       <c r="EN1" s="49"/>
-      <c r="EP1" s="108" t="s">
+      <c r="EP1" s="125" t="s">
         <v>223</v>
       </c>
-      <c r="EQ1" s="107"/>
-      <c r="ER1" s="107"/>
-      <c r="ES1" s="107"/>
-      <c r="ET1" s="107"/>
-      <c r="EU1" s="107"/>
+      <c r="EQ1" s="124"/>
+      <c r="ER1" s="124"/>
+      <c r="ES1" s="124"/>
+      <c r="ET1" s="124"/>
+      <c r="EU1" s="124"/>
       <c r="EV1" s="49"/>
       <c r="EW1" s="49"/>
       <c r="EX1" s="49"/>
@@ -17243,14 +17239,14 @@
       <c r="FD1" s="49"/>
     </row>
     <row r="2" spans="2:160" x14ac:dyDescent="0.25">
-      <c r="B2" s="108" t="s">
+      <c r="B2" s="125" t="s">
         <v>224</v>
       </c>
-      <c r="C2" s="107"/>
-      <c r="D2" s="107"/>
-      <c r="E2" s="107"/>
-      <c r="F2" s="107"/>
-      <c r="G2" s="107"/>
+      <c r="C2" s="124"/>
+      <c r="D2" s="124"/>
+      <c r="E2" s="124"/>
+      <c r="F2" s="124"/>
+      <c r="G2" s="124"/>
       <c r="H2" s="49"/>
       <c r="I2" s="49"/>
       <c r="J2" s="49"/>
@@ -17260,14 +17256,14 @@
       <c r="N2" s="49"/>
       <c r="O2" s="49"/>
       <c r="P2" s="49"/>
-      <c r="R2" s="111" t="s">
+      <c r="R2" s="128" t="s">
         <v>224</v>
       </c>
-      <c r="S2" s="112"/>
-      <c r="T2" s="112"/>
-      <c r="U2" s="112"/>
-      <c r="V2" s="112"/>
-      <c r="W2" s="112"/>
+      <c r="S2" s="129"/>
+      <c r="T2" s="129"/>
+      <c r="U2" s="129"/>
+      <c r="V2" s="129"/>
+      <c r="W2" s="129"/>
       <c r="X2" s="34"/>
       <c r="Y2" s="34"/>
       <c r="Z2" s="34"/>
@@ -17277,14 +17273,14 @@
       <c r="AD2" s="34"/>
       <c r="AE2" s="34"/>
       <c r="AF2" s="34"/>
-      <c r="AH2" s="108" t="s">
+      <c r="AH2" s="125" t="s">
         <v>224</v>
       </c>
-      <c r="AI2" s="107"/>
-      <c r="AJ2" s="107"/>
-      <c r="AK2" s="107"/>
-      <c r="AL2" s="107"/>
-      <c r="AM2" s="107"/>
+      <c r="AI2" s="124"/>
+      <c r="AJ2" s="124"/>
+      <c r="AK2" s="124"/>
+      <c r="AL2" s="124"/>
+      <c r="AM2" s="124"/>
       <c r="AN2" s="49"/>
       <c r="AO2" s="49"/>
       <c r="AP2" s="49"/>
@@ -17294,14 +17290,14 @@
       <c r="AT2" s="49"/>
       <c r="AU2" s="49"/>
       <c r="AV2" s="49"/>
-      <c r="AX2" s="108" t="s">
+      <c r="AX2" s="125" t="s">
         <v>224</v>
       </c>
-      <c r="AY2" s="107"/>
-      <c r="AZ2" s="107"/>
-      <c r="BA2" s="107"/>
-      <c r="BB2" s="107"/>
-      <c r="BC2" s="107"/>
+      <c r="AY2" s="124"/>
+      <c r="AZ2" s="124"/>
+      <c r="BA2" s="124"/>
+      <c r="BB2" s="124"/>
+      <c r="BC2" s="124"/>
       <c r="BD2" s="49"/>
       <c r="BE2" s="49"/>
       <c r="BF2" s="49"/>
@@ -17311,14 +17307,14 @@
       <c r="BJ2" s="49"/>
       <c r="BK2" s="49"/>
       <c r="BL2" s="49"/>
-      <c r="BN2" s="108" t="s">
+      <c r="BN2" s="125" t="s">
         <v>224</v>
       </c>
-      <c r="BO2" s="107"/>
-      <c r="BP2" s="107"/>
-      <c r="BQ2" s="107"/>
-      <c r="BR2" s="107"/>
-      <c r="BS2" s="107"/>
+      <c r="BO2" s="124"/>
+      <c r="BP2" s="124"/>
+      <c r="BQ2" s="124"/>
+      <c r="BR2" s="124"/>
+      <c r="BS2" s="124"/>
       <c r="BT2" s="49"/>
       <c r="BU2" s="49"/>
       <c r="BV2" s="49"/>
@@ -17329,14 +17325,14 @@
       <c r="CA2" s="49"/>
       <c r="CB2" s="49"/>
       <c r="CC2" s="34"/>
-      <c r="CD2" s="108" t="s">
+      <c r="CD2" s="125" t="s">
         <v>224</v>
       </c>
-      <c r="CE2" s="107"/>
-      <c r="CF2" s="107"/>
-      <c r="CG2" s="107"/>
-      <c r="CH2" s="107"/>
-      <c r="CI2" s="107"/>
+      <c r="CE2" s="124"/>
+      <c r="CF2" s="124"/>
+      <c r="CG2" s="124"/>
+      <c r="CH2" s="124"/>
+      <c r="CI2" s="124"/>
       <c r="CJ2" s="49"/>
       <c r="CK2" s="49"/>
       <c r="CL2" s="49"/>
@@ -17346,14 +17342,14 @@
       <c r="CP2" s="49"/>
       <c r="CQ2" s="49"/>
       <c r="CR2" s="49"/>
-      <c r="CT2" s="108" t="s">
+      <c r="CT2" s="125" t="s">
         <v>224</v>
       </c>
-      <c r="CU2" s="107"/>
-      <c r="CV2" s="107"/>
-      <c r="CW2" s="107"/>
-      <c r="CX2" s="107"/>
-      <c r="CY2" s="107"/>
+      <c r="CU2" s="124"/>
+      <c r="CV2" s="124"/>
+      <c r="CW2" s="124"/>
+      <c r="CX2" s="124"/>
+      <c r="CY2" s="124"/>
       <c r="CZ2" s="49"/>
       <c r="DA2" s="49"/>
       <c r="DB2" s="49"/>
@@ -17363,14 +17359,14 @@
       <c r="DF2" s="49"/>
       <c r="DG2" s="49"/>
       <c r="DH2" s="49"/>
-      <c r="DJ2" s="108" t="s">
+      <c r="DJ2" s="125" t="s">
         <v>224</v>
       </c>
-      <c r="DK2" s="107"/>
-      <c r="DL2" s="107"/>
-      <c r="DM2" s="107"/>
-      <c r="DN2" s="107"/>
-      <c r="DO2" s="107"/>
+      <c r="DK2" s="124"/>
+      <c r="DL2" s="124"/>
+      <c r="DM2" s="124"/>
+      <c r="DN2" s="124"/>
+      <c r="DO2" s="124"/>
       <c r="DP2" s="49"/>
       <c r="DQ2" s="49"/>
       <c r="DR2" s="49"/>
@@ -17380,14 +17376,14 @@
       <c r="DV2" s="49"/>
       <c r="DW2" s="49"/>
       <c r="DX2" s="49"/>
-      <c r="DZ2" s="108" t="s">
+      <c r="DZ2" s="125" t="s">
         <v>224</v>
       </c>
-      <c r="EA2" s="107"/>
-      <c r="EB2" s="107"/>
-      <c r="EC2" s="107"/>
-      <c r="ED2" s="107"/>
-      <c r="EE2" s="107"/>
+      <c r="EA2" s="124"/>
+      <c r="EB2" s="124"/>
+      <c r="EC2" s="124"/>
+      <c r="ED2" s="124"/>
+      <c r="EE2" s="124"/>
       <c r="EF2" s="49"/>
       <c r="EG2" s="49"/>
       <c r="EH2" s="49"/>
@@ -17397,14 +17393,14 @@
       <c r="EL2" s="49"/>
       <c r="EM2" s="49"/>
       <c r="EN2" s="49"/>
-      <c r="EP2" s="108" t="s">
+      <c r="EP2" s="125" t="s">
         <v>224</v>
       </c>
-      <c r="EQ2" s="107"/>
-      <c r="ER2" s="107"/>
-      <c r="ES2" s="107"/>
-      <c r="ET2" s="107"/>
-      <c r="EU2" s="107"/>
+      <c r="EQ2" s="124"/>
+      <c r="ER2" s="124"/>
+      <c r="ES2" s="124"/>
+      <c r="ET2" s="124"/>
+      <c r="EU2" s="124"/>
       <c r="EV2" s="49"/>
       <c r="EW2" s="49"/>
       <c r="EX2" s="49"/>
@@ -17416,12 +17412,12 @@
       <c r="FD2" s="49"/>
     </row>
     <row r="3" spans="2:160" x14ac:dyDescent="0.25">
-      <c r="B3" s="107"/>
-      <c r="C3" s="107"/>
-      <c r="D3" s="107"/>
-      <c r="E3" s="107"/>
-      <c r="F3" s="107"/>
-      <c r="G3" s="107"/>
+      <c r="B3" s="124"/>
+      <c r="C3" s="124"/>
+      <c r="D3" s="124"/>
+      <c r="E3" s="124"/>
+      <c r="F3" s="124"/>
+      <c r="G3" s="124"/>
       <c r="H3" s="49"/>
       <c r="I3" s="49"/>
       <c r="J3" s="49"/>
@@ -17431,12 +17427,12 @@
       <c r="N3" s="49"/>
       <c r="O3" s="49"/>
       <c r="P3" s="49"/>
-      <c r="R3" s="112"/>
-      <c r="S3" s="112"/>
-      <c r="T3" s="112"/>
-      <c r="U3" s="112"/>
-      <c r="V3" s="112"/>
-      <c r="W3" s="112"/>
+      <c r="R3" s="129"/>
+      <c r="S3" s="129"/>
+      <c r="T3" s="129"/>
+      <c r="U3" s="129"/>
+      <c r="V3" s="129"/>
+      <c r="W3" s="129"/>
       <c r="X3" s="34"/>
       <c r="Y3" s="34"/>
       <c r="Z3" s="34"/>
@@ -17446,12 +17442,12 @@
       <c r="AD3" s="34"/>
       <c r="AE3" s="34"/>
       <c r="AF3" s="34"/>
-      <c r="AH3" s="107"/>
-      <c r="AI3" s="107"/>
-      <c r="AJ3" s="107"/>
-      <c r="AK3" s="107"/>
-      <c r="AL3" s="107"/>
-      <c r="AM3" s="107"/>
+      <c r="AH3" s="124"/>
+      <c r="AI3" s="124"/>
+      <c r="AJ3" s="124"/>
+      <c r="AK3" s="124"/>
+      <c r="AL3" s="124"/>
+      <c r="AM3" s="124"/>
       <c r="AN3" s="49"/>
       <c r="AO3" s="49"/>
       <c r="AP3" s="49"/>
@@ -17461,12 +17457,12 @@
       <c r="AT3" s="49"/>
       <c r="AU3" s="49"/>
       <c r="AV3" s="49"/>
-      <c r="AX3" s="107"/>
-      <c r="AY3" s="107"/>
-      <c r="AZ3" s="107"/>
-      <c r="BA3" s="107"/>
-      <c r="BB3" s="107"/>
-      <c r="BC3" s="107"/>
+      <c r="AX3" s="124"/>
+      <c r="AY3" s="124"/>
+      <c r="AZ3" s="124"/>
+      <c r="BA3" s="124"/>
+      <c r="BB3" s="124"/>
+      <c r="BC3" s="124"/>
       <c r="BD3" s="49"/>
       <c r="BE3" s="49"/>
       <c r="BF3" s="49"/>
@@ -17476,12 +17472,12 @@
       <c r="BJ3" s="49"/>
       <c r="BK3" s="49"/>
       <c r="BL3" s="49"/>
-      <c r="BN3" s="107"/>
-      <c r="BO3" s="107"/>
-      <c r="BP3" s="107"/>
-      <c r="BQ3" s="107"/>
-      <c r="BR3" s="107"/>
-      <c r="BS3" s="107"/>
+      <c r="BN3" s="124"/>
+      <c r="BO3" s="124"/>
+      <c r="BP3" s="124"/>
+      <c r="BQ3" s="124"/>
+      <c r="BR3" s="124"/>
+      <c r="BS3" s="124"/>
       <c r="BT3" s="49"/>
       <c r="BU3" s="49"/>
       <c r="BV3" s="49"/>
@@ -17492,12 +17488,12 @@
       <c r="CA3" s="49"/>
       <c r="CB3" s="49"/>
       <c r="CC3" s="34"/>
-      <c r="CD3" s="107"/>
-      <c r="CE3" s="107"/>
-      <c r="CF3" s="107"/>
-      <c r="CG3" s="107"/>
-      <c r="CH3" s="107"/>
-      <c r="CI3" s="107"/>
+      <c r="CD3" s="124"/>
+      <c r="CE3" s="124"/>
+      <c r="CF3" s="124"/>
+      <c r="CG3" s="124"/>
+      <c r="CH3" s="124"/>
+      <c r="CI3" s="124"/>
       <c r="CJ3" s="49"/>
       <c r="CK3" s="49"/>
       <c r="CL3" s="49"/>
@@ -17507,12 +17503,12 @@
       <c r="CP3" s="49"/>
       <c r="CQ3" s="49"/>
       <c r="CR3" s="49"/>
-      <c r="CT3" s="107"/>
-      <c r="CU3" s="107"/>
-      <c r="CV3" s="107"/>
-      <c r="CW3" s="107"/>
-      <c r="CX3" s="107"/>
-      <c r="CY3" s="107"/>
+      <c r="CT3" s="124"/>
+      <c r="CU3" s="124"/>
+      <c r="CV3" s="124"/>
+      <c r="CW3" s="124"/>
+      <c r="CX3" s="124"/>
+      <c r="CY3" s="124"/>
       <c r="CZ3" s="49"/>
       <c r="DA3" s="49"/>
       <c r="DB3" s="49"/>
@@ -17522,12 +17518,12 @@
       <c r="DF3" s="49"/>
       <c r="DG3" s="49"/>
       <c r="DH3" s="49"/>
-      <c r="DJ3" s="107"/>
-      <c r="DK3" s="107"/>
-      <c r="DL3" s="107"/>
-      <c r="DM3" s="107"/>
-      <c r="DN3" s="107"/>
-      <c r="DO3" s="107"/>
+      <c r="DJ3" s="124"/>
+      <c r="DK3" s="124"/>
+      <c r="DL3" s="124"/>
+      <c r="DM3" s="124"/>
+      <c r="DN3" s="124"/>
+      <c r="DO3" s="124"/>
       <c r="DP3" s="49"/>
       <c r="DQ3" s="49"/>
       <c r="DR3" s="49"/>
@@ -17537,12 +17533,12 @@
       <c r="DV3" s="49"/>
       <c r="DW3" s="49"/>
       <c r="DX3" s="49"/>
-      <c r="DZ3" s="107"/>
-      <c r="EA3" s="107"/>
-      <c r="EB3" s="107"/>
-      <c r="EC3" s="107"/>
-      <c r="ED3" s="107"/>
-      <c r="EE3" s="107"/>
+      <c r="DZ3" s="124"/>
+      <c r="EA3" s="124"/>
+      <c r="EB3" s="124"/>
+      <c r="EC3" s="124"/>
+      <c r="ED3" s="124"/>
+      <c r="EE3" s="124"/>
       <c r="EF3" s="49"/>
       <c r="EG3" s="49"/>
       <c r="EH3" s="49"/>
@@ -17552,12 +17548,12 @@
       <c r="EL3" s="49"/>
       <c r="EM3" s="49"/>
       <c r="EN3" s="49"/>
-      <c r="EP3" s="107"/>
-      <c r="EQ3" s="107"/>
-      <c r="ER3" s="107"/>
-      <c r="ES3" s="107"/>
-      <c r="ET3" s="107"/>
-      <c r="EU3" s="107"/>
+      <c r="EP3" s="124"/>
+      <c r="EQ3" s="124"/>
+      <c r="ER3" s="124"/>
+      <c r="ES3" s="124"/>
+      <c r="ET3" s="124"/>
+      <c r="EU3" s="124"/>
       <c r="EV3" s="49"/>
       <c r="EW3" s="49"/>
       <c r="EX3" s="49"/>
@@ -17572,13 +17568,13 @@
       <c r="B4" s="50" t="s">
         <v>146</v>
       </c>
-      <c r="C4" s="109" t="s">
+      <c r="C4" s="126" t="s">
         <v>170</v>
       </c>
-      <c r="D4" s="107"/>
-      <c r="E4" s="107"/>
-      <c r="F4" s="107"/>
-      <c r="G4" s="107"/>
+      <c r="D4" s="124"/>
+      <c r="E4" s="124"/>
+      <c r="F4" s="124"/>
+      <c r="G4" s="124"/>
       <c r="H4" s="49"/>
       <c r="I4" s="49"/>
       <c r="J4" s="49"/>
@@ -17591,13 +17587,13 @@
       <c r="R4" s="35" t="s">
         <v>146</v>
       </c>
-      <c r="S4" s="114" t="s">
+      <c r="S4" s="131" t="s">
         <v>225</v>
       </c>
-      <c r="T4" s="112"/>
-      <c r="U4" s="112"/>
-      <c r="V4" s="112"/>
-      <c r="W4" s="112"/>
+      <c r="T4" s="129"/>
+      <c r="U4" s="129"/>
+      <c r="V4" s="129"/>
+      <c r="W4" s="129"/>
       <c r="X4" s="34"/>
       <c r="Y4" s="34"/>
       <c r="Z4" s="34"/>
@@ -17610,13 +17606,13 @@
       <c r="AH4" s="50" t="s">
         <v>146</v>
       </c>
-      <c r="AI4" s="109" t="s">
+      <c r="AI4" s="126" t="s">
         <v>147</v>
       </c>
-      <c r="AJ4" s="107"/>
-      <c r="AK4" s="107"/>
-      <c r="AL4" s="107"/>
-      <c r="AM4" s="107"/>
+      <c r="AJ4" s="124"/>
+      <c r="AK4" s="124"/>
+      <c r="AL4" s="124"/>
+      <c r="AM4" s="124"/>
       <c r="AN4" s="49"/>
       <c r="AO4" s="49"/>
       <c r="AP4" s="49"/>
@@ -17629,13 +17625,13 @@
       <c r="AX4" s="50" t="s">
         <v>146</v>
       </c>
-      <c r="AY4" s="109" t="s">
+      <c r="AY4" s="126" t="s">
         <v>171</v>
       </c>
-      <c r="AZ4" s="107"/>
-      <c r="BA4" s="107"/>
-      <c r="BB4" s="107"/>
-      <c r="BC4" s="107"/>
+      <c r="AZ4" s="124"/>
+      <c r="BA4" s="124"/>
+      <c r="BB4" s="124"/>
+      <c r="BC4" s="124"/>
       <c r="BD4" s="49"/>
       <c r="BE4" s="49"/>
       <c r="BF4" s="49"/>
@@ -17648,13 +17644,13 @@
       <c r="BN4" s="50" t="s">
         <v>146</v>
       </c>
-      <c r="BO4" s="109" t="s">
+      <c r="BO4" s="126" t="s">
         <v>244</v>
       </c>
-      <c r="BP4" s="107"/>
-      <c r="BQ4" s="107"/>
-      <c r="BR4" s="107"/>
-      <c r="BS4" s="107"/>
+      <c r="BP4" s="124"/>
+      <c r="BQ4" s="124"/>
+      <c r="BR4" s="124"/>
+      <c r="BS4" s="124"/>
       <c r="BT4" s="49"/>
       <c r="BU4" s="49"/>
       <c r="BV4" s="49"/>
@@ -17668,13 +17664,13 @@
       <c r="CD4" s="50" t="s">
         <v>146</v>
       </c>
-      <c r="CE4" s="109" t="s">
+      <c r="CE4" s="126" t="s">
         <v>241</v>
       </c>
-      <c r="CF4" s="107"/>
-      <c r="CG4" s="107"/>
-      <c r="CH4" s="107"/>
-      <c r="CI4" s="107"/>
+      <c r="CF4" s="124"/>
+      <c r="CG4" s="124"/>
+      <c r="CH4" s="124"/>
+      <c r="CI4" s="124"/>
       <c r="CJ4" s="49"/>
       <c r="CK4" s="49"/>
       <c r="CL4" s="49"/>
@@ -17687,13 +17683,13 @@
       <c r="CT4" s="50" t="s">
         <v>146</v>
       </c>
-      <c r="CU4" s="109" t="s">
+      <c r="CU4" s="126" t="s">
         <v>257</v>
       </c>
-      <c r="CV4" s="107"/>
-      <c r="CW4" s="107"/>
-      <c r="CX4" s="107"/>
-      <c r="CY4" s="107"/>
+      <c r="CV4" s="124"/>
+      <c r="CW4" s="124"/>
+      <c r="CX4" s="124"/>
+      <c r="CY4" s="124"/>
       <c r="CZ4" s="49"/>
       <c r="DA4" s="49"/>
       <c r="DB4" s="49"/>
@@ -17706,13 +17702,13 @@
       <c r="DJ4" s="50" t="s">
         <v>146</v>
       </c>
-      <c r="DK4" s="109" t="s">
+      <c r="DK4" s="126" t="s">
         <v>231</v>
       </c>
-      <c r="DL4" s="107"/>
-      <c r="DM4" s="107"/>
-      <c r="DN4" s="107"/>
-      <c r="DO4" s="107"/>
+      <c r="DL4" s="124"/>
+      <c r="DM4" s="124"/>
+      <c r="DN4" s="124"/>
+      <c r="DO4" s="124"/>
       <c r="DP4" s="49"/>
       <c r="DQ4" s="49"/>
       <c r="DR4" s="49"/>
@@ -17725,13 +17721,13 @@
       <c r="DZ4" s="50" t="s">
         <v>146</v>
       </c>
-      <c r="EA4" s="109" t="s">
+      <c r="EA4" s="126" t="s">
         <v>248</v>
       </c>
-      <c r="EB4" s="107"/>
-      <c r="EC4" s="107"/>
-      <c r="ED4" s="107"/>
-      <c r="EE4" s="107"/>
+      <c r="EB4" s="124"/>
+      <c r="EC4" s="124"/>
+      <c r="ED4" s="124"/>
+      <c r="EE4" s="124"/>
       <c r="EF4" s="49"/>
       <c r="EG4" s="49"/>
       <c r="EH4" s="49"/>
@@ -17744,13 +17740,13 @@
       <c r="EP4" s="50" t="s">
         <v>146</v>
       </c>
-      <c r="EQ4" s="109" t="s">
+      <c r="EQ4" s="126" t="s">
         <v>236</v>
       </c>
-      <c r="ER4" s="107"/>
-      <c r="ES4" s="107"/>
-      <c r="ET4" s="107"/>
-      <c r="EU4" s="107"/>
+      <c r="ER4" s="124"/>
+      <c r="ES4" s="124"/>
+      <c r="ET4" s="124"/>
+      <c r="EU4" s="124"/>
       <c r="EV4" s="49"/>
       <c r="EW4" s="49"/>
       <c r="EX4" s="49"/>
@@ -17762,14 +17758,14 @@
       <c r="FD4" s="49"/>
     </row>
     <row r="5" spans="2:160" x14ac:dyDescent="0.25">
-      <c r="B5" s="110" t="s">
+      <c r="B5" s="127" t="s">
         <v>31</v>
       </c>
-      <c r="C5" s="107"/>
-      <c r="D5" s="107"/>
-      <c r="E5" s="107"/>
-      <c r="F5" s="107"/>
-      <c r="G5" s="107"/>
+      <c r="C5" s="124"/>
+      <c r="D5" s="124"/>
+      <c r="E5" s="124"/>
+      <c r="F5" s="124"/>
+      <c r="G5" s="124"/>
       <c r="H5" s="49"/>
       <c r="I5" s="49"/>
       <c r="J5" s="49"/>
@@ -17779,14 +17775,14 @@
       <c r="N5" s="49"/>
       <c r="O5" s="49"/>
       <c r="P5" s="49"/>
-      <c r="R5" s="115" t="s">
+      <c r="R5" s="132" t="s">
         <v>31</v>
       </c>
-      <c r="S5" s="112"/>
-      <c r="T5" s="112"/>
-      <c r="U5" s="112"/>
-      <c r="V5" s="112"/>
-      <c r="W5" s="112"/>
+      <c r="S5" s="129"/>
+      <c r="T5" s="129"/>
+      <c r="U5" s="129"/>
+      <c r="V5" s="129"/>
+      <c r="W5" s="129"/>
       <c r="X5" s="34"/>
       <c r="Y5" s="34"/>
       <c r="Z5" s="34"/>
@@ -17796,14 +17792,14 @@
       <c r="AD5" s="34"/>
       <c r="AE5" s="34"/>
       <c r="AF5" s="34"/>
-      <c r="AH5" s="110" t="s">
+      <c r="AH5" s="127" t="s">
         <v>31</v>
       </c>
-      <c r="AI5" s="107"/>
-      <c r="AJ5" s="107"/>
-      <c r="AK5" s="107"/>
-      <c r="AL5" s="107"/>
-      <c r="AM5" s="107"/>
+      <c r="AI5" s="124"/>
+      <c r="AJ5" s="124"/>
+      <c r="AK5" s="124"/>
+      <c r="AL5" s="124"/>
+      <c r="AM5" s="124"/>
       <c r="AN5" s="49"/>
       <c r="AO5" s="49"/>
       <c r="AP5" s="49"/>
@@ -17813,14 +17809,14 @@
       <c r="AT5" s="49"/>
       <c r="AU5" s="49"/>
       <c r="AV5" s="49"/>
-      <c r="AX5" s="110" t="s">
+      <c r="AX5" s="127" t="s">
         <v>31</v>
       </c>
-      <c r="AY5" s="107"/>
-      <c r="AZ5" s="107"/>
-      <c r="BA5" s="107"/>
-      <c r="BB5" s="107"/>
-      <c r="BC5" s="107"/>
+      <c r="AY5" s="124"/>
+      <c r="AZ5" s="124"/>
+      <c r="BA5" s="124"/>
+      <c r="BB5" s="124"/>
+      <c r="BC5" s="124"/>
       <c r="BD5" s="49"/>
       <c r="BE5" s="49"/>
       <c r="BF5" s="49"/>
@@ -17830,14 +17826,14 @@
       <c r="BJ5" s="49"/>
       <c r="BK5" s="49"/>
       <c r="BL5" s="49"/>
-      <c r="BN5" s="110" t="s">
+      <c r="BN5" s="127" t="s">
         <v>31</v>
       </c>
-      <c r="BO5" s="107"/>
-      <c r="BP5" s="107"/>
-      <c r="BQ5" s="107"/>
-      <c r="BR5" s="107"/>
-      <c r="BS5" s="107"/>
+      <c r="BO5" s="124"/>
+      <c r="BP5" s="124"/>
+      <c r="BQ5" s="124"/>
+      <c r="BR5" s="124"/>
+      <c r="BS5" s="124"/>
       <c r="BT5" s="49"/>
       <c r="BU5" s="49"/>
       <c r="BV5" s="49"/>
@@ -17848,14 +17844,14 @@
       <c r="CA5" s="49"/>
       <c r="CB5" s="49"/>
       <c r="CC5" s="34"/>
-      <c r="CD5" s="110" t="s">
+      <c r="CD5" s="127" t="s">
         <v>31</v>
       </c>
-      <c r="CE5" s="107"/>
-      <c r="CF5" s="107"/>
-      <c r="CG5" s="107"/>
-      <c r="CH5" s="107"/>
-      <c r="CI5" s="107"/>
+      <c r="CE5" s="124"/>
+      <c r="CF5" s="124"/>
+      <c r="CG5" s="124"/>
+      <c r="CH5" s="124"/>
+      <c r="CI5" s="124"/>
       <c r="CJ5" s="49"/>
       <c r="CK5" s="49"/>
       <c r="CL5" s="49"/>
@@ -17865,14 +17861,14 @@
       <c r="CP5" s="49"/>
       <c r="CQ5" s="49"/>
       <c r="CR5" s="49"/>
-      <c r="CT5" s="110" t="s">
+      <c r="CT5" s="127" t="s">
         <v>31</v>
       </c>
-      <c r="CU5" s="107"/>
-      <c r="CV5" s="107"/>
-      <c r="CW5" s="107"/>
-      <c r="CX5" s="107"/>
-      <c r="CY5" s="107"/>
+      <c r="CU5" s="124"/>
+      <c r="CV5" s="124"/>
+      <c r="CW5" s="124"/>
+      <c r="CX5" s="124"/>
+      <c r="CY5" s="124"/>
       <c r="CZ5" s="49"/>
       <c r="DA5" s="49"/>
       <c r="DB5" s="49"/>
@@ -17882,14 +17878,14 @@
       <c r="DF5" s="49"/>
       <c r="DG5" s="49"/>
       <c r="DH5" s="49"/>
-      <c r="DJ5" s="110" t="s">
+      <c r="DJ5" s="127" t="s">
         <v>31</v>
       </c>
-      <c r="DK5" s="107"/>
-      <c r="DL5" s="107"/>
-      <c r="DM5" s="107"/>
-      <c r="DN5" s="107"/>
-      <c r="DO5" s="107"/>
+      <c r="DK5" s="124"/>
+      <c r="DL5" s="124"/>
+      <c r="DM5" s="124"/>
+      <c r="DN5" s="124"/>
+      <c r="DO5" s="124"/>
       <c r="DP5" s="49"/>
       <c r="DQ5" s="49"/>
       <c r="DR5" s="49"/>
@@ -17899,14 +17895,14 @@
       <c r="DV5" s="49"/>
       <c r="DW5" s="49"/>
       <c r="DX5" s="49"/>
-      <c r="DZ5" s="110" t="s">
+      <c r="DZ5" s="127" t="s">
         <v>31</v>
       </c>
-      <c r="EA5" s="107"/>
-      <c r="EB5" s="107"/>
-      <c r="EC5" s="107"/>
-      <c r="ED5" s="107"/>
-      <c r="EE5" s="107"/>
+      <c r="EA5" s="124"/>
+      <c r="EB5" s="124"/>
+      <c r="EC5" s="124"/>
+      <c r="ED5" s="124"/>
+      <c r="EE5" s="124"/>
       <c r="EF5" s="49"/>
       <c r="EG5" s="49"/>
       <c r="EH5" s="49"/>
@@ -17916,14 +17912,14 @@
       <c r="EL5" s="49"/>
       <c r="EM5" s="49"/>
       <c r="EN5" s="49"/>
-      <c r="EP5" s="110" t="s">
+      <c r="EP5" s="127" t="s">
         <v>31</v>
       </c>
-      <c r="EQ5" s="107"/>
-      <c r="ER5" s="107"/>
-      <c r="ES5" s="107"/>
-      <c r="ET5" s="107"/>
-      <c r="EU5" s="107"/>
+      <c r="EQ5" s="124"/>
+      <c r="ER5" s="124"/>
+      <c r="ES5" s="124"/>
+      <c r="ET5" s="124"/>
+      <c r="EU5" s="124"/>
       <c r="EV5" s="49"/>
       <c r="EW5" s="49"/>
       <c r="EX5" s="49"/>
@@ -17938,13 +17934,13 @@
       <c r="B6" s="50" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="109" t="s">
+      <c r="C6" s="126" t="s">
         <v>172</v>
       </c>
-      <c r="D6" s="107"/>
-      <c r="E6" s="107"/>
-      <c r="F6" s="107"/>
-      <c r="G6" s="107"/>
+      <c r="D6" s="124"/>
+      <c r="E6" s="124"/>
+      <c r="F6" s="124"/>
+      <c r="G6" s="124"/>
       <c r="H6" s="49"/>
       <c r="I6" s="49"/>
       <c r="J6" s="49"/>
@@ -17957,13 +17953,13 @@
       <c r="R6" s="35" t="s">
         <v>32</v>
       </c>
-      <c r="S6" s="114" t="s">
+      <c r="S6" s="131" t="s">
         <v>226</v>
       </c>
-      <c r="T6" s="112"/>
-      <c r="U6" s="112"/>
-      <c r="V6" s="112"/>
-      <c r="W6" s="112"/>
+      <c r="T6" s="129"/>
+      <c r="U6" s="129"/>
+      <c r="V6" s="129"/>
+      <c r="W6" s="129"/>
       <c r="X6" s="34"/>
       <c r="Y6" s="34"/>
       <c r="Z6" s="34"/>
@@ -17976,13 +17972,13 @@
       <c r="AH6" s="50" t="s">
         <v>32</v>
       </c>
-      <c r="AI6" s="109" t="s">
+      <c r="AI6" s="126" t="s">
         <v>148</v>
       </c>
-      <c r="AJ6" s="107"/>
-      <c r="AK6" s="107"/>
-      <c r="AL6" s="107"/>
-      <c r="AM6" s="107"/>
+      <c r="AJ6" s="124"/>
+      <c r="AK6" s="124"/>
+      <c r="AL6" s="124"/>
+      <c r="AM6" s="124"/>
       <c r="AN6" s="49"/>
       <c r="AO6" s="49"/>
       <c r="AP6" s="49"/>
@@ -17995,13 +17991,13 @@
       <c r="AX6" s="50" t="s">
         <v>32</v>
       </c>
-      <c r="AY6" s="109" t="s">
+      <c r="AY6" s="126" t="s">
         <v>173</v>
       </c>
-      <c r="AZ6" s="107"/>
-      <c r="BA6" s="107"/>
-      <c r="BB6" s="107"/>
-      <c r="BC6" s="107"/>
+      <c r="AZ6" s="124"/>
+      <c r="BA6" s="124"/>
+      <c r="BB6" s="124"/>
+      <c r="BC6" s="124"/>
       <c r="BD6" s="49"/>
       <c r="BE6" s="49"/>
       <c r="BF6" s="49"/>
@@ -18014,13 +18010,13 @@
       <c r="BN6" s="50" t="s">
         <v>32</v>
       </c>
-      <c r="BO6" s="109" t="s">
+      <c r="BO6" s="126" t="s">
         <v>245</v>
       </c>
-      <c r="BP6" s="107"/>
-      <c r="BQ6" s="107"/>
-      <c r="BR6" s="107"/>
-      <c r="BS6" s="107"/>
+      <c r="BP6" s="124"/>
+      <c r="BQ6" s="124"/>
+      <c r="BR6" s="124"/>
+      <c r="BS6" s="124"/>
       <c r="BT6" s="49"/>
       <c r="BU6" s="49"/>
       <c r="BV6" s="49"/>
@@ -18033,13 +18029,13 @@
       <c r="CD6" s="50" t="s">
         <v>32</v>
       </c>
-      <c r="CE6" s="109" t="s">
+      <c r="CE6" s="126" t="s">
         <v>242</v>
       </c>
-      <c r="CF6" s="107"/>
-      <c r="CG6" s="107"/>
-      <c r="CH6" s="107"/>
-      <c r="CI6" s="107"/>
+      <c r="CF6" s="124"/>
+      <c r="CG6" s="124"/>
+      <c r="CH6" s="124"/>
+      <c r="CI6" s="124"/>
       <c r="CJ6" s="49"/>
       <c r="CK6" s="49"/>
       <c r="CL6" s="49"/>
@@ -18052,13 +18048,13 @@
       <c r="CT6" s="50" t="s">
         <v>32</v>
       </c>
-      <c r="CU6" s="109" t="s">
+      <c r="CU6" s="126" t="s">
         <v>258</v>
       </c>
-      <c r="CV6" s="107"/>
-      <c r="CW6" s="107"/>
-      <c r="CX6" s="107"/>
-      <c r="CY6" s="107"/>
+      <c r="CV6" s="124"/>
+      <c r="CW6" s="124"/>
+      <c r="CX6" s="124"/>
+      <c r="CY6" s="124"/>
       <c r="CZ6" s="49"/>
       <c r="DA6" s="49"/>
       <c r="DB6" s="49"/>
@@ -18071,13 +18067,13 @@
       <c r="DJ6" s="50" t="s">
         <v>32</v>
       </c>
-      <c r="DK6" s="109" t="s">
+      <c r="DK6" s="126" t="s">
         <v>232</v>
       </c>
-      <c r="DL6" s="107"/>
-      <c r="DM6" s="107"/>
-      <c r="DN6" s="107"/>
-      <c r="DO6" s="107"/>
+      <c r="DL6" s="124"/>
+      <c r="DM6" s="124"/>
+      <c r="DN6" s="124"/>
+      <c r="DO6" s="124"/>
       <c r="DP6" s="49"/>
       <c r="DQ6" s="49"/>
       <c r="DR6" s="49"/>
@@ -18090,13 +18086,13 @@
       <c r="DZ6" s="50" t="s">
         <v>32</v>
       </c>
-      <c r="EA6" s="109" t="s">
+      <c r="EA6" s="126" t="s">
         <v>249</v>
       </c>
-      <c r="EB6" s="107"/>
-      <c r="EC6" s="107"/>
-      <c r="ED6" s="107"/>
-      <c r="EE6" s="107"/>
+      <c r="EB6" s="124"/>
+      <c r="EC6" s="124"/>
+      <c r="ED6" s="124"/>
+      <c r="EE6" s="124"/>
       <c r="EF6" s="49"/>
       <c r="EG6" s="49"/>
       <c r="EH6" s="49"/>
@@ -18109,13 +18105,13 @@
       <c r="EP6" s="50" t="s">
         <v>32</v>
       </c>
-      <c r="EQ6" s="109" t="s">
+      <c r="EQ6" s="126" t="s">
         <v>237</v>
       </c>
-      <c r="ER6" s="107"/>
-      <c r="ES6" s="107"/>
-      <c r="ET6" s="107"/>
-      <c r="EU6" s="107"/>
+      <c r="ER6" s="124"/>
+      <c r="ES6" s="124"/>
+      <c r="ET6" s="124"/>
+      <c r="EU6" s="124"/>
       <c r="EV6" s="49"/>
       <c r="EW6" s="49"/>
       <c r="EX6" s="49"/>
@@ -18130,13 +18126,13 @@
       <c r="B7" s="50" t="s">
         <v>33</v>
       </c>
-      <c r="C7" s="109" t="s">
+      <c r="C7" s="126" t="s">
         <v>34</v>
       </c>
-      <c r="D7" s="107"/>
-      <c r="E7" s="107"/>
-      <c r="F7" s="107"/>
-      <c r="G7" s="107"/>
+      <c r="D7" s="124"/>
+      <c r="E7" s="124"/>
+      <c r="F7" s="124"/>
+      <c r="G7" s="124"/>
       <c r="H7" s="49"/>
       <c r="I7" s="49"/>
       <c r="J7" s="49"/>
@@ -18149,13 +18145,13 @@
       <c r="R7" s="35" t="s">
         <v>33</v>
       </c>
-      <c r="S7" s="114" t="s">
+      <c r="S7" s="131" t="s">
         <v>34</v>
       </c>
-      <c r="T7" s="112"/>
-      <c r="U7" s="112"/>
-      <c r="V7" s="112"/>
-      <c r="W7" s="112"/>
+      <c r="T7" s="129"/>
+      <c r="U7" s="129"/>
+      <c r="V7" s="129"/>
+      <c r="W7" s="129"/>
       <c r="X7" s="34"/>
       <c r="Y7" s="34"/>
       <c r="Z7" s="34"/>
@@ -18168,13 +18164,13 @@
       <c r="AH7" s="50" t="s">
         <v>33</v>
       </c>
-      <c r="AI7" s="109" t="s">
+      <c r="AI7" s="126" t="s">
         <v>34</v>
       </c>
-      <c r="AJ7" s="107"/>
-      <c r="AK7" s="107"/>
-      <c r="AL7" s="107"/>
-      <c r="AM7" s="107"/>
+      <c r="AJ7" s="124"/>
+      <c r="AK7" s="124"/>
+      <c r="AL7" s="124"/>
+      <c r="AM7" s="124"/>
       <c r="AN7" s="49"/>
       <c r="AO7" s="49"/>
       <c r="AP7" s="49"/>
@@ -18187,13 +18183,13 @@
       <c r="AX7" s="50" t="s">
         <v>33</v>
       </c>
-      <c r="AY7" s="109" t="s">
+      <c r="AY7" s="126" t="s">
         <v>34</v>
       </c>
-      <c r="AZ7" s="107"/>
-      <c r="BA7" s="107"/>
-      <c r="BB7" s="107"/>
-      <c r="BC7" s="107"/>
+      <c r="AZ7" s="124"/>
+      <c r="BA7" s="124"/>
+      <c r="BB7" s="124"/>
+      <c r="BC7" s="124"/>
       <c r="BD7" s="49"/>
       <c r="BE7" s="49"/>
       <c r="BF7" s="49"/>
@@ -18206,13 +18202,13 @@
       <c r="BN7" s="50" t="s">
         <v>33</v>
       </c>
-      <c r="BO7" s="109" t="s">
+      <c r="BO7" s="126" t="s">
         <v>34</v>
       </c>
-      <c r="BP7" s="107"/>
-      <c r="BQ7" s="107"/>
-      <c r="BR7" s="107"/>
-      <c r="BS7" s="107"/>
+      <c r="BP7" s="124"/>
+      <c r="BQ7" s="124"/>
+      <c r="BR7" s="124"/>
+      <c r="BS7" s="124"/>
       <c r="BT7" s="49"/>
       <c r="BU7" s="49"/>
       <c r="BV7" s="49"/>
@@ -18225,13 +18221,13 @@
       <c r="CD7" s="50" t="s">
         <v>33</v>
       </c>
-      <c r="CE7" s="109" t="s">
+      <c r="CE7" s="126" t="s">
         <v>34</v>
       </c>
-      <c r="CF7" s="107"/>
-      <c r="CG7" s="107"/>
-      <c r="CH7" s="107"/>
-      <c r="CI7" s="107"/>
+      <c r="CF7" s="124"/>
+      <c r="CG7" s="124"/>
+      <c r="CH7" s="124"/>
+      <c r="CI7" s="124"/>
       <c r="CJ7" s="49"/>
       <c r="CK7" s="49"/>
       <c r="CL7" s="49"/>
@@ -18244,13 +18240,13 @@
       <c r="CT7" s="50" t="s">
         <v>33</v>
       </c>
-      <c r="CU7" s="109" t="s">
+      <c r="CU7" s="126" t="s">
         <v>34</v>
       </c>
-      <c r="CV7" s="107"/>
-      <c r="CW7" s="107"/>
-      <c r="CX7" s="107"/>
-      <c r="CY7" s="107"/>
+      <c r="CV7" s="124"/>
+      <c r="CW7" s="124"/>
+      <c r="CX7" s="124"/>
+      <c r="CY7" s="124"/>
       <c r="CZ7" s="49"/>
       <c r="DA7" s="49"/>
       <c r="DB7" s="49"/>
@@ -18263,13 +18259,13 @@
       <c r="DJ7" s="50" t="s">
         <v>33</v>
       </c>
-      <c r="DK7" s="109" t="s">
+      <c r="DK7" s="126" t="s">
         <v>34</v>
       </c>
-      <c r="DL7" s="107"/>
-      <c r="DM7" s="107"/>
-      <c r="DN7" s="107"/>
-      <c r="DO7" s="107"/>
+      <c r="DL7" s="124"/>
+      <c r="DM7" s="124"/>
+      <c r="DN7" s="124"/>
+      <c r="DO7" s="124"/>
       <c r="DP7" s="49"/>
       <c r="DQ7" s="49"/>
       <c r="DR7" s="49"/>
@@ -18282,13 +18278,13 @@
       <c r="DZ7" s="50" t="s">
         <v>33</v>
       </c>
-      <c r="EA7" s="109" t="s">
+      <c r="EA7" s="126" t="s">
         <v>34</v>
       </c>
-      <c r="EB7" s="107"/>
-      <c r="EC7" s="107"/>
-      <c r="ED7" s="107"/>
-      <c r="EE7" s="107"/>
+      <c r="EB7" s="124"/>
+      <c r="EC7" s="124"/>
+      <c r="ED7" s="124"/>
+      <c r="EE7" s="124"/>
       <c r="EF7" s="49"/>
       <c r="EG7" s="49"/>
       <c r="EH7" s="49"/>
@@ -18301,13 +18297,13 @@
       <c r="EP7" s="50" t="s">
         <v>33</v>
       </c>
-      <c r="EQ7" s="109" t="s">
+      <c r="EQ7" s="126" t="s">
         <v>34</v>
       </c>
-      <c r="ER7" s="107"/>
-      <c r="ES7" s="107"/>
-      <c r="ET7" s="107"/>
-      <c r="EU7" s="107"/>
+      <c r="ER7" s="124"/>
+      <c r="ES7" s="124"/>
+      <c r="ET7" s="124"/>
+      <c r="EU7" s="124"/>
       <c r="EV7" s="49"/>
       <c r="EW7" s="49"/>
       <c r="EX7" s="49"/>
@@ -18322,18 +18318,18 @@
       <c r="B8" s="50" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="109" t="s">
+      <c r="C8" s="126" t="s">
         <v>144</v>
       </c>
-      <c r="D8" s="107"/>
-      <c r="E8" s="107"/>
-      <c r="F8" s="107"/>
-      <c r="G8" s="107"/>
+      <c r="D8" s="124"/>
+      <c r="E8" s="124"/>
+      <c r="F8" s="124"/>
+      <c r="G8" s="124"/>
       <c r="H8" s="49"/>
-      <c r="I8" s="116" t="s">
+      <c r="I8" s="98" t="s">
         <v>409</v>
       </c>
-      <c r="J8" s="117">
+      <c r="J8" s="99">
         <f>(N43/N13)^(1/30)-1</f>
         <v>2.3977134838169212E-2</v>
       </c>
@@ -18346,18 +18342,18 @@
       <c r="R8" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="S8" s="120" t="s">
+      <c r="S8" s="131" t="s">
         <v>227</v>
       </c>
-      <c r="T8" s="121"/>
-      <c r="U8" s="121"/>
-      <c r="V8" s="121"/>
-      <c r="W8" s="121"/>
+      <c r="T8" s="129"/>
+      <c r="U8" s="129"/>
+      <c r="V8" s="129"/>
+      <c r="W8" s="129"/>
       <c r="X8" s="55"/>
-      <c r="Y8" s="116" t="s">
+      <c r="Y8" s="98" t="s">
         <v>409</v>
       </c>
-      <c r="Z8" s="117">
+      <c r="Z8" s="99">
         <f>(X43/X13)^(1/30)-1</f>
         <v>2.0736944174645666E-2</v>
       </c>
@@ -18370,18 +18366,18 @@
       <c r="AH8" s="50" t="s">
         <v>35</v>
       </c>
-      <c r="AI8" s="109" t="s">
+      <c r="AI8" s="126" t="s">
         <v>149</v>
       </c>
-      <c r="AJ8" s="107"/>
-      <c r="AK8" s="107"/>
-      <c r="AL8" s="107"/>
-      <c r="AM8" s="107"/>
+      <c r="AJ8" s="124"/>
+      <c r="AK8" s="124"/>
+      <c r="AL8" s="124"/>
+      <c r="AM8" s="124"/>
       <c r="AN8" s="49"/>
-      <c r="AO8" s="116" t="s">
+      <c r="AO8" s="98" t="s">
         <v>409</v>
       </c>
-      <c r="AP8" s="117">
+      <c r="AP8" s="99">
         <f>(AT43/AT13)^(1/30)-1</f>
         <v>3.5117348400309334E-2</v>
       </c>
@@ -18394,18 +18390,18 @@
       <c r="AX8" s="50" t="s">
         <v>35</v>
       </c>
-      <c r="AY8" s="109" t="s">
+      <c r="AY8" s="126" t="s">
         <v>174</v>
       </c>
-      <c r="AZ8" s="107"/>
-      <c r="BA8" s="107"/>
-      <c r="BB8" s="107"/>
-      <c r="BC8" s="107"/>
+      <c r="AZ8" s="124"/>
+      <c r="BA8" s="124"/>
+      <c r="BB8" s="124"/>
+      <c r="BC8" s="124"/>
       <c r="BD8" s="49"/>
-      <c r="BE8" s="116" t="s">
+      <c r="BE8" s="98" t="s">
         <v>409</v>
       </c>
-      <c r="BF8" s="117">
+      <c r="BF8" s="99">
         <f>(BJ43/BJ13)^(1/30)-1</f>
         <v>2.9548225004298212E-2</v>
       </c>
@@ -18418,18 +18414,18 @@
       <c r="BN8" s="50" t="s">
         <v>35</v>
       </c>
-      <c r="BO8" s="109" t="s">
+      <c r="BO8" s="126" t="s">
         <v>246</v>
       </c>
-      <c r="BP8" s="107"/>
-      <c r="BQ8" s="107"/>
-      <c r="BR8" s="107"/>
-      <c r="BS8" s="107"/>
+      <c r="BP8" s="124"/>
+      <c r="BQ8" s="124"/>
+      <c r="BR8" s="124"/>
+      <c r="BS8" s="124"/>
       <c r="BT8" s="49"/>
-      <c r="BU8" s="116" t="s">
+      <c r="BU8" s="98" t="s">
         <v>409</v>
       </c>
-      <c r="BV8" s="117">
+      <c r="BV8" s="99">
         <f>(BZ29/BZ13)^(1/16)-1</f>
         <v>6.3201478284775625E-3</v>
       </c>
@@ -18444,18 +18440,18 @@
       <c r="CD8" s="50" t="s">
         <v>35</v>
       </c>
-      <c r="CE8" s="109" t="s">
+      <c r="CE8" s="126" t="s">
         <v>243</v>
       </c>
-      <c r="CF8" s="107"/>
-      <c r="CG8" s="107"/>
-      <c r="CH8" s="107"/>
-      <c r="CI8" s="107"/>
+      <c r="CF8" s="124"/>
+      <c r="CG8" s="124"/>
+      <c r="CH8" s="124"/>
+      <c r="CI8" s="124"/>
       <c r="CJ8" s="49"/>
-      <c r="CK8" s="116" t="s">
+      <c r="CK8" s="98" t="s">
         <v>409</v>
       </c>
-      <c r="CL8" s="117">
+      <c r="CL8" s="99">
         <f>(CP43/CP13)^(1/30)-1</f>
         <v>2.5219757035239265E-2</v>
       </c>
@@ -18468,18 +18464,18 @@
       <c r="CT8" s="50" t="s">
         <v>35</v>
       </c>
-      <c r="CU8" s="109" t="s">
+      <c r="CU8" s="126" t="s">
         <v>259</v>
       </c>
-      <c r="CV8" s="107"/>
-      <c r="CW8" s="107"/>
-      <c r="CX8" s="107"/>
-      <c r="CY8" s="107"/>
+      <c r="CV8" s="124"/>
+      <c r="CW8" s="124"/>
+      <c r="CX8" s="124"/>
+      <c r="CY8" s="124"/>
       <c r="CZ8" s="49"/>
-      <c r="DA8" s="116" t="s">
+      <c r="DA8" s="98" t="s">
         <v>409</v>
       </c>
-      <c r="DB8" s="117">
+      <c r="DB8" s="99">
         <f>(DF42/DF13)^(1/29)-1</f>
         <v>5.2913605158896315E-2</v>
       </c>
@@ -18493,18 +18489,18 @@
       <c r="DJ8" s="50" t="s">
         <v>35</v>
       </c>
-      <c r="DK8" s="109" t="s">
+      <c r="DK8" s="126" t="s">
         <v>233</v>
       </c>
-      <c r="DL8" s="107"/>
-      <c r="DM8" s="107"/>
-      <c r="DN8" s="107"/>
-      <c r="DO8" s="107"/>
+      <c r="DL8" s="124"/>
+      <c r="DM8" s="124"/>
+      <c r="DN8" s="124"/>
+      <c r="DO8" s="124"/>
       <c r="DP8" s="49"/>
-      <c r="DQ8" s="116" t="s">
+      <c r="DQ8" s="98" t="s">
         <v>409</v>
       </c>
-      <c r="DR8" s="117">
+      <c r="DR8" s="99">
         <f>(DS42/DS14)^(1/28)-1</f>
         <v>5.2018836646548605E-2</v>
       </c>
@@ -18517,18 +18513,18 @@
       <c r="DZ8" s="50" t="s">
         <v>35</v>
       </c>
-      <c r="EA8" s="109" t="s">
+      <c r="EA8" s="126" t="s">
         <v>139</v>
       </c>
-      <c r="EB8" s="107"/>
-      <c r="EC8" s="107"/>
-      <c r="ED8" s="107"/>
-      <c r="EE8" s="107"/>
+      <c r="EB8" s="124"/>
+      <c r="EC8" s="124"/>
+      <c r="ED8" s="124"/>
+      <c r="EE8" s="124"/>
       <c r="EF8" s="49"/>
-      <c r="EG8" s="116" t="s">
+      <c r="EG8" s="98" t="s">
         <v>409</v>
       </c>
-      <c r="EH8" s="117">
+      <c r="EH8" s="99">
         <f>(EL43/EL13)^(1/30)-1</f>
         <v>5.2900906226266198E-2</v>
       </c>
@@ -18541,18 +18537,18 @@
       <c r="EP8" s="50" t="s">
         <v>35</v>
       </c>
-      <c r="EQ8" s="109" t="s">
+      <c r="EQ8" s="126" t="s">
         <v>238</v>
       </c>
-      <c r="ER8" s="107"/>
-      <c r="ES8" s="107"/>
-      <c r="ET8" s="107"/>
-      <c r="EU8" s="107"/>
+      <c r="ER8" s="124"/>
+      <c r="ES8" s="124"/>
+      <c r="ET8" s="124"/>
+      <c r="EU8" s="124"/>
       <c r="EV8" s="49"/>
-      <c r="EW8" s="116" t="s">
+      <c r="EW8" s="98" t="s">
         <v>409</v>
       </c>
-      <c r="EX8" s="117">
+      <c r="EX8" s="99">
         <f>(FB29/FB14)^(1/15)-1</f>
         <v>7.3233117948781068E-3</v>
       </c>
@@ -18567,18 +18563,18 @@
       <c r="B9" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="109" t="s">
+      <c r="C9" s="126" t="s">
         <v>150</v>
       </c>
-      <c r="D9" s="107"/>
-      <c r="E9" s="107"/>
-      <c r="F9" s="107"/>
-      <c r="G9" s="107"/>
+      <c r="D9" s="124"/>
+      <c r="E9" s="124"/>
+      <c r="F9" s="124"/>
+      <c r="G9" s="124"/>
       <c r="H9" s="49"/>
-      <c r="I9" s="116" t="s">
+      <c r="I9" s="98" t="s">
         <v>410</v>
       </c>
-      <c r="J9" s="118"/>
+      <c r="J9" s="100"/>
       <c r="K9" s="49"/>
       <c r="L9" s="49"/>
       <c r="M9" s="49"/>
@@ -18588,18 +18584,18 @@
       <c r="R9" s="35" t="s">
         <v>36</v>
       </c>
-      <c r="S9" s="114" t="s">
+      <c r="S9" s="131" t="s">
         <v>228</v>
       </c>
-      <c r="T9" s="112"/>
-      <c r="U9" s="112"/>
-      <c r="V9" s="112"/>
-      <c r="W9" s="112"/>
+      <c r="T9" s="129"/>
+      <c r="U9" s="129"/>
+      <c r="V9" s="129"/>
+      <c r="W9" s="129"/>
       <c r="X9" s="34"/>
-      <c r="Y9" s="116" t="s">
+      <c r="Y9" s="98" t="s">
         <v>410</v>
       </c>
-      <c r="Z9" s="119"/>
+      <c r="Z9" s="101"/>
       <c r="AA9" s="34"/>
       <c r="AB9" s="34"/>
       <c r="AC9" s="34"/>
@@ -18609,18 +18605,18 @@
       <c r="AH9" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="AI9" s="109" t="s">
+      <c r="AI9" s="126" t="s">
         <v>150</v>
       </c>
-      <c r="AJ9" s="107"/>
-      <c r="AK9" s="107"/>
-      <c r="AL9" s="107"/>
-      <c r="AM9" s="107"/>
+      <c r="AJ9" s="124"/>
+      <c r="AK9" s="124"/>
+      <c r="AL9" s="124"/>
+      <c r="AM9" s="124"/>
       <c r="AN9" s="49"/>
-      <c r="AO9" s="116" t="s">
+      <c r="AO9" s="98" t="s">
         <v>410</v>
       </c>
-      <c r="AP9" s="118"/>
+      <c r="AP9" s="100"/>
       <c r="AQ9" s="49"/>
       <c r="AR9" s="49"/>
       <c r="AS9" s="49"/>
@@ -18630,18 +18626,18 @@
       <c r="AX9" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="AY9" s="109" t="s">
+      <c r="AY9" s="126" t="s">
         <v>150</v>
       </c>
-      <c r="AZ9" s="107"/>
-      <c r="BA9" s="107"/>
-      <c r="BB9" s="107"/>
-      <c r="BC9" s="107"/>
+      <c r="AZ9" s="124"/>
+      <c r="BA9" s="124"/>
+      <c r="BB9" s="124"/>
+      <c r="BC9" s="124"/>
       <c r="BD9" s="49"/>
-      <c r="BE9" s="116" t="s">
+      <c r="BE9" s="98" t="s">
         <v>410</v>
       </c>
-      <c r="BF9" s="118"/>
+      <c r="BF9" s="100"/>
       <c r="BG9" s="49"/>
       <c r="BH9" s="49"/>
       <c r="BI9" s="49"/>
@@ -18651,18 +18647,18 @@
       <c r="BN9" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="BO9" s="109" t="s">
+      <c r="BO9" s="126" t="s">
         <v>239</v>
       </c>
-      <c r="BP9" s="107"/>
-      <c r="BQ9" s="107"/>
-      <c r="BR9" s="107"/>
-      <c r="BS9" s="107"/>
+      <c r="BP9" s="124"/>
+      <c r="BQ9" s="124"/>
+      <c r="BR9" s="124"/>
+      <c r="BS9" s="124"/>
       <c r="BT9" s="49"/>
-      <c r="BU9" s="116" t="s">
+      <c r="BU9" s="98" t="s">
         <v>410</v>
       </c>
-      <c r="BV9" s="118"/>
+      <c r="BV9" s="100"/>
       <c r="BW9" s="49"/>
       <c r="BX9" s="49"/>
       <c r="BY9" s="49"/>
@@ -18672,18 +18668,18 @@
       <c r="CD9" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="CE9" s="109" t="s">
+      <c r="CE9" s="126" t="s">
         <v>150</v>
       </c>
-      <c r="CF9" s="107"/>
-      <c r="CG9" s="107"/>
-      <c r="CH9" s="107"/>
-      <c r="CI9" s="107"/>
+      <c r="CF9" s="124"/>
+      <c r="CG9" s="124"/>
+      <c r="CH9" s="124"/>
+      <c r="CI9" s="124"/>
       <c r="CJ9" s="49"/>
-      <c r="CK9" s="116" t="s">
+      <c r="CK9" s="98" t="s">
         <v>410</v>
       </c>
-      <c r="CL9" s="118"/>
+      <c r="CL9" s="100"/>
       <c r="CM9" s="49"/>
       <c r="CN9" s="49"/>
       <c r="CO9" s="49"/>
@@ -18693,18 +18689,18 @@
       <c r="CT9" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="CU9" s="109" t="s">
+      <c r="CU9" s="126" t="s">
         <v>234</v>
       </c>
-      <c r="CV9" s="107"/>
-      <c r="CW9" s="107"/>
-      <c r="CX9" s="107"/>
-      <c r="CY9" s="107"/>
+      <c r="CV9" s="124"/>
+      <c r="CW9" s="124"/>
+      <c r="CX9" s="124"/>
+      <c r="CY9" s="124"/>
       <c r="CZ9" s="49"/>
-      <c r="DA9" s="116" t="s">
+      <c r="DA9" s="98" t="s">
         <v>410</v>
       </c>
-      <c r="DB9" s="118"/>
+      <c r="DB9" s="100"/>
       <c r="DC9" s="49"/>
       <c r="DD9" s="49"/>
       <c r="DE9" s="49"/>
@@ -18714,18 +18710,18 @@
       <c r="DJ9" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="DK9" s="109" t="s">
+      <c r="DK9" s="126" t="s">
         <v>234</v>
       </c>
-      <c r="DL9" s="107"/>
-      <c r="DM9" s="107"/>
-      <c r="DN9" s="107"/>
-      <c r="DO9" s="107"/>
+      <c r="DL9" s="124"/>
+      <c r="DM9" s="124"/>
+      <c r="DN9" s="124"/>
+      <c r="DO9" s="124"/>
       <c r="DP9" s="49"/>
-      <c r="DQ9" s="116" t="s">
+      <c r="DQ9" s="98" t="s">
         <v>410</v>
       </c>
-      <c r="DR9" s="118"/>
+      <c r="DR9" s="100"/>
       <c r="DS9" s="49"/>
       <c r="DT9" s="49"/>
       <c r="DU9" s="49"/>
@@ -18735,18 +18731,18 @@
       <c r="DZ9" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="EA9" s="109" t="s">
+      <c r="EA9" s="126" t="s">
         <v>228</v>
       </c>
-      <c r="EB9" s="107"/>
-      <c r="EC9" s="107"/>
-      <c r="ED9" s="107"/>
-      <c r="EE9" s="107"/>
+      <c r="EB9" s="124"/>
+      <c r="EC9" s="124"/>
+      <c r="ED9" s="124"/>
+      <c r="EE9" s="124"/>
       <c r="EF9" s="49"/>
-      <c r="EG9" s="116" t="s">
+      <c r="EG9" s="98" t="s">
         <v>410</v>
       </c>
-      <c r="EH9" s="118"/>
+      <c r="EH9" s="100"/>
       <c r="EI9" s="49"/>
       <c r="EJ9" s="49"/>
       <c r="EK9" s="49"/>
@@ -18756,18 +18752,18 @@
       <c r="EP9" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="EQ9" s="109" t="s">
+      <c r="EQ9" s="126" t="s">
         <v>239</v>
       </c>
-      <c r="ER9" s="107"/>
-      <c r="ES9" s="107"/>
-      <c r="ET9" s="107"/>
-      <c r="EU9" s="107"/>
+      <c r="ER9" s="124"/>
+      <c r="ES9" s="124"/>
+      <c r="ET9" s="124"/>
+      <c r="EU9" s="124"/>
       <c r="EV9" s="49"/>
-      <c r="EW9" s="116" t="s">
+      <c r="EW9" s="98" t="s">
         <v>410</v>
       </c>
-      <c r="EX9" s="118"/>
+      <c r="EX9" s="100"/>
       <c r="EY9" s="49"/>
       <c r="EZ9" s="49"/>
       <c r="FA9" s="49"/>
@@ -18779,13 +18775,13 @@
       <c r="B10" s="50" t="s">
         <v>229</v>
       </c>
-      <c r="C10" s="106" t="s">
+      <c r="C10" s="123" t="s">
         <v>230</v>
       </c>
-      <c r="D10" s="107"/>
-      <c r="E10" s="107"/>
-      <c r="F10" s="107"/>
-      <c r="G10" s="107"/>
+      <c r="D10" s="124"/>
+      <c r="E10" s="124"/>
+      <c r="F10" s="124"/>
+      <c r="G10" s="124"/>
       <c r="H10" s="49"/>
       <c r="I10" s="49"/>
       <c r="J10" s="49"/>
@@ -18798,13 +18794,13 @@
       <c r="R10" s="35" t="s">
         <v>229</v>
       </c>
-      <c r="S10" s="113" t="s">
+      <c r="S10" s="130" t="s">
         <v>230</v>
       </c>
-      <c r="T10" s="112"/>
-      <c r="U10" s="112"/>
-      <c r="V10" s="112"/>
-      <c r="W10" s="112"/>
+      <c r="T10" s="129"/>
+      <c r="U10" s="129"/>
+      <c r="V10" s="129"/>
+      <c r="W10" s="129"/>
       <c r="X10" s="34"/>
       <c r="Y10" s="34"/>
       <c r="Z10" s="34"/>
@@ -18817,13 +18813,13 @@
       <c r="AH10" s="50" t="s">
         <v>229</v>
       </c>
-      <c r="AI10" s="106" t="s">
+      <c r="AI10" s="123" t="s">
         <v>230</v>
       </c>
-      <c r="AJ10" s="107"/>
-      <c r="AK10" s="107"/>
-      <c r="AL10" s="107"/>
-      <c r="AM10" s="107"/>
+      <c r="AJ10" s="124"/>
+      <c r="AK10" s="124"/>
+      <c r="AL10" s="124"/>
+      <c r="AM10" s="124"/>
       <c r="AN10" s="49"/>
       <c r="AO10" s="49"/>
       <c r="AP10" s="49"/>
@@ -18836,13 +18832,13 @@
       <c r="AX10" s="50" t="s">
         <v>229</v>
       </c>
-      <c r="AY10" s="106" t="s">
+      <c r="AY10" s="123" t="s">
         <v>230</v>
       </c>
-      <c r="AZ10" s="107"/>
-      <c r="BA10" s="107"/>
-      <c r="BB10" s="107"/>
-      <c r="BC10" s="107"/>
+      <c r="AZ10" s="124"/>
+      <c r="BA10" s="124"/>
+      <c r="BB10" s="124"/>
+      <c r="BC10" s="124"/>
       <c r="BD10" s="49"/>
       <c r="BE10" s="49"/>
       <c r="BF10" s="49"/>
@@ -18855,13 +18851,13 @@
       <c r="BN10" s="50" t="s">
         <v>229</v>
       </c>
-      <c r="BO10" s="106" t="s">
+      <c r="BO10" s="123" t="s">
         <v>240</v>
       </c>
-      <c r="BP10" s="107"/>
-      <c r="BQ10" s="107"/>
-      <c r="BR10" s="107"/>
-      <c r="BS10" s="107"/>
+      <c r="BP10" s="124"/>
+      <c r="BQ10" s="124"/>
+      <c r="BR10" s="124"/>
+      <c r="BS10" s="124"/>
       <c r="BT10" s="49"/>
       <c r="BU10" s="49"/>
       <c r="BV10" s="49"/>
@@ -18874,13 +18870,13 @@
       <c r="CD10" s="50" t="s">
         <v>229</v>
       </c>
-      <c r="CE10" s="106" t="s">
+      <c r="CE10" s="123" t="s">
         <v>230</v>
       </c>
-      <c r="CF10" s="107"/>
-      <c r="CG10" s="107"/>
-      <c r="CH10" s="107"/>
-      <c r="CI10" s="107"/>
+      <c r="CF10" s="124"/>
+      <c r="CG10" s="124"/>
+      <c r="CH10" s="124"/>
+      <c r="CI10" s="124"/>
       <c r="CJ10" s="49"/>
       <c r="CK10" s="49"/>
       <c r="CL10" s="49"/>
@@ -18893,13 +18889,13 @@
       <c r="CT10" s="50" t="s">
         <v>229</v>
       </c>
-      <c r="CU10" s="106" t="s">
+      <c r="CU10" s="123" t="s">
         <v>235</v>
       </c>
-      <c r="CV10" s="107"/>
-      <c r="CW10" s="107"/>
-      <c r="CX10" s="107"/>
-      <c r="CY10" s="107"/>
+      <c r="CV10" s="124"/>
+      <c r="CW10" s="124"/>
+      <c r="CX10" s="124"/>
+      <c r="CY10" s="124"/>
       <c r="CZ10" s="49"/>
       <c r="DA10" s="49"/>
       <c r="DB10" s="49"/>
@@ -18912,13 +18908,13 @@
       <c r="DJ10" s="50" t="s">
         <v>229</v>
       </c>
-      <c r="DK10" s="106" t="s">
+      <c r="DK10" s="123" t="s">
         <v>235</v>
       </c>
-      <c r="DL10" s="107"/>
-      <c r="DM10" s="107"/>
-      <c r="DN10" s="107"/>
-      <c r="DO10" s="107"/>
+      <c r="DL10" s="124"/>
+      <c r="DM10" s="124"/>
+      <c r="DN10" s="124"/>
+      <c r="DO10" s="124"/>
       <c r="DP10" s="49"/>
       <c r="DQ10" s="49"/>
       <c r="DR10" s="49"/>
@@ -18931,13 +18927,13 @@
       <c r="DZ10" s="50" t="s">
         <v>229</v>
       </c>
-      <c r="EA10" s="106" t="s">
+      <c r="EA10" s="123" t="s">
         <v>230</v>
       </c>
-      <c r="EB10" s="107"/>
-      <c r="EC10" s="107"/>
-      <c r="ED10" s="107"/>
-      <c r="EE10" s="107"/>
+      <c r="EB10" s="124"/>
+      <c r="EC10" s="124"/>
+      <c r="ED10" s="124"/>
+      <c r="EE10" s="124"/>
       <c r="EF10" s="49"/>
       <c r="EG10" s="49"/>
       <c r="EH10" s="49"/>
@@ -18950,13 +18946,13 @@
       <c r="EP10" s="50" t="s">
         <v>229</v>
       </c>
-      <c r="EQ10" s="106" t="s">
+      <c r="EQ10" s="123" t="s">
         <v>240</v>
       </c>
-      <c r="ER10" s="107"/>
-      <c r="ES10" s="107"/>
-      <c r="ET10" s="107"/>
-      <c r="EU10" s="107"/>
+      <c r="ER10" s="124"/>
+      <c r="ES10" s="124"/>
+      <c r="ET10" s="124"/>
+      <c r="EU10" s="124"/>
       <c r="EV10" s="49"/>
       <c r="EW10" s="49"/>
       <c r="EX10" s="49"/>
@@ -31140,14 +31136,14 @@
       <c r="EN43" s="49"/>
     </row>
     <row r="45" spans="2:144" x14ac:dyDescent="0.25">
-      <c r="R45" s="108" t="s">
+      <c r="R45" s="125" t="s">
         <v>223</v>
       </c>
-      <c r="S45" s="107"/>
-      <c r="T45" s="107"/>
-      <c r="U45" s="107"/>
-      <c r="V45" s="107"/>
-      <c r="W45" s="107"/>
+      <c r="S45" s="124"/>
+      <c r="T45" s="124"/>
+      <c r="U45" s="124"/>
+      <c r="V45" s="124"/>
+      <c r="W45" s="124"/>
       <c r="X45" s="49"/>
       <c r="Y45" s="49"/>
       <c r="Z45" s="49"/>
@@ -31159,14 +31155,14 @@
       <c r="AF45" s="49"/>
     </row>
     <row r="46" spans="2:144" x14ac:dyDescent="0.25">
-      <c r="R46" s="108" t="s">
+      <c r="R46" s="125" t="s">
         <v>224</v>
       </c>
-      <c r="S46" s="107"/>
-      <c r="T46" s="107"/>
-      <c r="U46" s="107"/>
-      <c r="V46" s="107"/>
-      <c r="W46" s="107"/>
+      <c r="S46" s="124"/>
+      <c r="T46" s="124"/>
+      <c r="U46" s="124"/>
+      <c r="V46" s="124"/>
+      <c r="W46" s="124"/>
       <c r="X46" s="49"/>
       <c r="Y46" s="49"/>
       <c r="Z46" s="49"/>
@@ -31178,12 +31174,12 @@
       <c r="AF46" s="49"/>
     </row>
     <row r="47" spans="2:144" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="R47" s="107"/>
-      <c r="S47" s="107"/>
-      <c r="T47" s="107"/>
-      <c r="U47" s="107"/>
-      <c r="V47" s="107"/>
-      <c r="W47" s="107"/>
+      <c r="R47" s="124"/>
+      <c r="S47" s="124"/>
+      <c r="T47" s="124"/>
+      <c r="U47" s="124"/>
+      <c r="V47" s="124"/>
+      <c r="W47" s="124"/>
       <c r="X47" s="49"/>
       <c r="Y47" s="49"/>
       <c r="Z47" s="49"/>
@@ -31198,13 +31194,13 @@
       <c r="R48" s="50" t="s">
         <v>146</v>
       </c>
-      <c r="S48" s="109" t="s">
+      <c r="S48" s="126" t="s">
         <v>225</v>
       </c>
-      <c r="T48" s="107"/>
-      <c r="U48" s="107"/>
-      <c r="V48" s="107"/>
-      <c r="W48" s="107"/>
+      <c r="T48" s="124"/>
+      <c r="U48" s="124"/>
+      <c r="V48" s="124"/>
+      <c r="W48" s="124"/>
       <c r="X48" s="49"/>
       <c r="Y48" s="49"/>
       <c r="Z48" s="49"/>
@@ -31216,14 +31212,14 @@
       <c r="AF48" s="49"/>
     </row>
     <row r="49" spans="18:32" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="R49" s="110" t="s">
+      <c r="R49" s="127" t="s">
         <v>31</v>
       </c>
-      <c r="S49" s="107"/>
-      <c r="T49" s="107"/>
-      <c r="U49" s="107"/>
-      <c r="V49" s="107"/>
-      <c r="W49" s="107"/>
+      <c r="S49" s="124"/>
+      <c r="T49" s="124"/>
+      <c r="U49" s="124"/>
+      <c r="V49" s="124"/>
+      <c r="W49" s="124"/>
       <c r="X49" s="49"/>
       <c r="Y49" s="49"/>
       <c r="Z49" s="49"/>
@@ -31238,13 +31234,13 @@
       <c r="R50" s="50" t="s">
         <v>32</v>
       </c>
-      <c r="S50" s="109" t="s">
+      <c r="S50" s="126" t="s">
         <v>226</v>
       </c>
-      <c r="T50" s="107"/>
-      <c r="U50" s="107"/>
-      <c r="V50" s="107"/>
-      <c r="W50" s="107"/>
+      <c r="T50" s="124"/>
+      <c r="U50" s="124"/>
+      <c r="V50" s="124"/>
+      <c r="W50" s="124"/>
       <c r="X50" s="49"/>
       <c r="Y50" s="49"/>
       <c r="Z50" s="49"/>
@@ -31259,13 +31255,13 @@
       <c r="R51" s="50" t="s">
         <v>33</v>
       </c>
-      <c r="S51" s="109" t="s">
+      <c r="S51" s="126" t="s">
         <v>34</v>
       </c>
-      <c r="T51" s="107"/>
-      <c r="U51" s="107"/>
-      <c r="V51" s="107"/>
-      <c r="W51" s="107"/>
+      <c r="T51" s="124"/>
+      <c r="U51" s="124"/>
+      <c r="V51" s="124"/>
+      <c r="W51" s="124"/>
       <c r="X51" s="49"/>
       <c r="Y51" s="49"/>
       <c r="Z51" s="49"/>
@@ -31280,13 +31276,13 @@
       <c r="R52" s="50" t="s">
         <v>35</v>
       </c>
-      <c r="S52" s="109" t="s">
+      <c r="S52" s="126" t="s">
         <v>227</v>
       </c>
-      <c r="T52" s="107"/>
-      <c r="U52" s="107"/>
-      <c r="V52" s="107"/>
-      <c r="W52" s="107"/>
+      <c r="T52" s="124"/>
+      <c r="U52" s="124"/>
+      <c r="V52" s="124"/>
+      <c r="W52" s="124"/>
       <c r="X52" s="49"/>
       <c r="Y52" s="49"/>
       <c r="Z52" s="49"/>
@@ -31301,13 +31297,13 @@
       <c r="R53" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="S53" s="109" t="s">
+      <c r="S53" s="126" t="s">
         <v>228</v>
       </c>
-      <c r="T53" s="107"/>
-      <c r="U53" s="107"/>
-      <c r="V53" s="107"/>
-      <c r="W53" s="107"/>
+      <c r="T53" s="124"/>
+      <c r="U53" s="124"/>
+      <c r="V53" s="124"/>
+      <c r="W53" s="124"/>
       <c r="X53" s="49"/>
       <c r="Y53" s="49"/>
       <c r="Z53" s="49"/>
@@ -31322,13 +31318,13 @@
       <c r="R54" s="50" t="s">
         <v>229</v>
       </c>
-      <c r="S54" s="106" t="s">
+      <c r="S54" s="123" t="s">
         <v>230</v>
       </c>
-      <c r="T54" s="107"/>
-      <c r="U54" s="107"/>
-      <c r="V54" s="107"/>
-      <c r="W54" s="107"/>
+      <c r="T54" s="124"/>
+      <c r="U54" s="124"/>
+      <c r="V54" s="124"/>
+      <c r="W54" s="124"/>
       <c r="X54" s="49"/>
       <c r="Y54" s="49"/>
       <c r="Z54" s="49"/>
@@ -32709,38 +32705,60 @@
     </row>
   </sheetData>
   <mergeCells count="110">
-    <mergeCell ref="EA10:EE10"/>
-    <mergeCell ref="DJ1:DO1"/>
-    <mergeCell ref="DJ2:DO2"/>
-    <mergeCell ref="DJ3:DO3"/>
-    <mergeCell ref="DK4:DO4"/>
-    <mergeCell ref="DK6:DO6"/>
-    <mergeCell ref="DK7:DO7"/>
-    <mergeCell ref="DK8:DO8"/>
-    <mergeCell ref="DK9:DO9"/>
-    <mergeCell ref="DJ5:DO5"/>
-    <mergeCell ref="DK10:DO10"/>
-    <mergeCell ref="DZ1:EE1"/>
-    <mergeCell ref="DZ2:EE2"/>
-    <mergeCell ref="DZ3:EE3"/>
-    <mergeCell ref="EA4:EE4"/>
-    <mergeCell ref="DZ5:EE5"/>
-    <mergeCell ref="EA6:EE6"/>
-    <mergeCell ref="EA7:EE7"/>
-    <mergeCell ref="EA8:EE8"/>
-    <mergeCell ref="EA9:EE9"/>
-    <mergeCell ref="CE9:CI9"/>
-    <mergeCell ref="BO10:BS10"/>
-    <mergeCell ref="CU6:CY6"/>
-    <mergeCell ref="CU7:CY7"/>
-    <mergeCell ref="CU8:CY8"/>
-    <mergeCell ref="CU9:CY9"/>
-    <mergeCell ref="CU10:CY10"/>
-    <mergeCell ref="CT1:CY1"/>
-    <mergeCell ref="CT2:CY2"/>
-    <mergeCell ref="CT3:CY3"/>
-    <mergeCell ref="CU4:CY4"/>
-    <mergeCell ref="CT5:CY5"/>
+    <mergeCell ref="EQ10:EU10"/>
+    <mergeCell ref="EP1:EU1"/>
+    <mergeCell ref="EP2:EU2"/>
+    <mergeCell ref="EP3:EU3"/>
+    <mergeCell ref="EQ4:EU4"/>
+    <mergeCell ref="EP5:EU5"/>
+    <mergeCell ref="EQ6:EU6"/>
+    <mergeCell ref="EQ7:EU7"/>
+    <mergeCell ref="EQ8:EU8"/>
+    <mergeCell ref="EQ9:EU9"/>
+    <mergeCell ref="C10:G10"/>
+    <mergeCell ref="R1:W1"/>
+    <mergeCell ref="B1:G1"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="C9:G9"/>
+    <mergeCell ref="S10:W10"/>
+    <mergeCell ref="S7:W7"/>
+    <mergeCell ref="S8:W8"/>
+    <mergeCell ref="S9:W9"/>
+    <mergeCell ref="S4:W4"/>
+    <mergeCell ref="R5:W5"/>
+    <mergeCell ref="S6:W6"/>
+    <mergeCell ref="R2:W2"/>
+    <mergeCell ref="R3:W3"/>
+    <mergeCell ref="AY10:BC10"/>
+    <mergeCell ref="S53:W53"/>
+    <mergeCell ref="S54:W54"/>
+    <mergeCell ref="AH1:AM1"/>
+    <mergeCell ref="AH2:AM2"/>
+    <mergeCell ref="AH3:AM3"/>
+    <mergeCell ref="AI4:AM4"/>
+    <mergeCell ref="AH5:AM5"/>
+    <mergeCell ref="AI6:AM6"/>
+    <mergeCell ref="AI7:AM7"/>
+    <mergeCell ref="AI8:AM8"/>
+    <mergeCell ref="AI9:AM9"/>
+    <mergeCell ref="AI10:AM10"/>
+    <mergeCell ref="R45:W45"/>
+    <mergeCell ref="R46:W46"/>
+    <mergeCell ref="R47:W47"/>
+    <mergeCell ref="S48:W48"/>
+    <mergeCell ref="R49:W49"/>
+    <mergeCell ref="S50:W50"/>
+    <mergeCell ref="S51:W51"/>
+    <mergeCell ref="S52:W52"/>
+    <mergeCell ref="AX1:BC1"/>
+    <mergeCell ref="AX2:BC2"/>
+    <mergeCell ref="AX3:BC3"/>
     <mergeCell ref="AY4:BC4"/>
     <mergeCell ref="AX5:BC5"/>
     <mergeCell ref="AY6:BC6"/>
@@ -32765,60 +32783,38 @@
     <mergeCell ref="CE6:CI6"/>
     <mergeCell ref="CE7:CI7"/>
     <mergeCell ref="CE8:CI8"/>
-    <mergeCell ref="AY10:BC10"/>
-    <mergeCell ref="S53:W53"/>
-    <mergeCell ref="S54:W54"/>
-    <mergeCell ref="AH1:AM1"/>
-    <mergeCell ref="AH2:AM2"/>
-    <mergeCell ref="AH3:AM3"/>
-    <mergeCell ref="AI4:AM4"/>
-    <mergeCell ref="AH5:AM5"/>
-    <mergeCell ref="AI6:AM6"/>
-    <mergeCell ref="AI7:AM7"/>
-    <mergeCell ref="AI8:AM8"/>
-    <mergeCell ref="AI9:AM9"/>
-    <mergeCell ref="AI10:AM10"/>
-    <mergeCell ref="R45:W45"/>
-    <mergeCell ref="R46:W46"/>
-    <mergeCell ref="R47:W47"/>
-    <mergeCell ref="S48:W48"/>
-    <mergeCell ref="R49:W49"/>
-    <mergeCell ref="S50:W50"/>
-    <mergeCell ref="S51:W51"/>
-    <mergeCell ref="S52:W52"/>
-    <mergeCell ref="AX1:BC1"/>
-    <mergeCell ref="AX2:BC2"/>
-    <mergeCell ref="AX3:BC3"/>
-    <mergeCell ref="C10:G10"/>
-    <mergeCell ref="R1:W1"/>
-    <mergeCell ref="B1:G1"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="B3:G3"/>
-    <mergeCell ref="C4:G4"/>
-    <mergeCell ref="B5:G5"/>
-    <mergeCell ref="C6:G6"/>
-    <mergeCell ref="C7:G7"/>
-    <mergeCell ref="C8:G8"/>
-    <mergeCell ref="C9:G9"/>
-    <mergeCell ref="S10:W10"/>
-    <mergeCell ref="S7:W7"/>
-    <mergeCell ref="S8:W8"/>
-    <mergeCell ref="S9:W9"/>
-    <mergeCell ref="S4:W4"/>
-    <mergeCell ref="R5:W5"/>
-    <mergeCell ref="S6:W6"/>
-    <mergeCell ref="R2:W2"/>
-    <mergeCell ref="R3:W3"/>
-    <mergeCell ref="EQ10:EU10"/>
-    <mergeCell ref="EP1:EU1"/>
-    <mergeCell ref="EP2:EU2"/>
-    <mergeCell ref="EP3:EU3"/>
-    <mergeCell ref="EQ4:EU4"/>
-    <mergeCell ref="EP5:EU5"/>
-    <mergeCell ref="EQ6:EU6"/>
-    <mergeCell ref="EQ7:EU7"/>
-    <mergeCell ref="EQ8:EU8"/>
-    <mergeCell ref="EQ9:EU9"/>
+    <mergeCell ref="CE9:CI9"/>
+    <mergeCell ref="BO10:BS10"/>
+    <mergeCell ref="CU6:CY6"/>
+    <mergeCell ref="CU7:CY7"/>
+    <mergeCell ref="CU8:CY8"/>
+    <mergeCell ref="CU9:CY9"/>
+    <mergeCell ref="CU10:CY10"/>
+    <mergeCell ref="CT1:CY1"/>
+    <mergeCell ref="CT2:CY2"/>
+    <mergeCell ref="CT3:CY3"/>
+    <mergeCell ref="CU4:CY4"/>
+    <mergeCell ref="CT5:CY5"/>
+    <mergeCell ref="EA10:EE10"/>
+    <mergeCell ref="DJ1:DO1"/>
+    <mergeCell ref="DJ2:DO2"/>
+    <mergeCell ref="DJ3:DO3"/>
+    <mergeCell ref="DK4:DO4"/>
+    <mergeCell ref="DK6:DO6"/>
+    <mergeCell ref="DK7:DO7"/>
+    <mergeCell ref="DK8:DO8"/>
+    <mergeCell ref="DK9:DO9"/>
+    <mergeCell ref="DJ5:DO5"/>
+    <mergeCell ref="DK10:DO10"/>
+    <mergeCell ref="DZ1:EE1"/>
+    <mergeCell ref="DZ2:EE2"/>
+    <mergeCell ref="DZ3:EE3"/>
+    <mergeCell ref="EA4:EE4"/>
+    <mergeCell ref="DZ5:EE5"/>
+    <mergeCell ref="EA6:EE6"/>
+    <mergeCell ref="EA7:EE7"/>
+    <mergeCell ref="EA8:EE8"/>
+    <mergeCell ref="EA9:EE9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>